<commit_message>
corrected time difference error
</commit_message>
<xml_diff>
--- a/results/interim_results/pmf_results/stationary_pmf_bs_fpeak.xlsx
+++ b/results/interim_results/pmf_results/stationary_pmf_bs_fpeak.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lf649/git_repos/active/thriveair_analysis/results/interim_results/pmf_results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECBC1E7-5643-D54B-967D-3C7916C6FAB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236507C2-1582-DB4B-9A78-338C1E5B9818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5680" yWindow="980" windowWidth="21800" windowHeight="11220" activeTab="5" xr2:uid="{09D946F0-50DC-4E8E-81BA-F953608CE5F7}"/>
+    <workbookView xWindow="6560" yWindow="1300" windowWidth="15840" windowHeight="12520" activeTab="4" xr2:uid="{55429072-0D44-41EB-8E51-4D66B05BF716}"/>
   </bookViews>
   <sheets>
     <sheet name="Factor 1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="Factor 3" sheetId="3" r:id="rId3"/>
     <sheet name="Factor 4" sheetId="4" r:id="rId4"/>
     <sheet name="Factor 5" sheetId="5" r:id="rId5"/>
-    <sheet name="Key" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="35">
   <si>
     <t>Species</t>
   </si>
@@ -147,30 +146,6 @@
   <si>
     <t>BS 95th pct</t>
   </si>
-  <si>
-    <t>Factor</t>
-  </si>
-  <si>
-    <t>% mass</t>
-  </si>
-  <si>
-    <t>Interpretation</t>
-  </si>
-  <si>
-    <t>Background/legacy</t>
-  </si>
-  <si>
-    <t>Gasoline evaporation</t>
-  </si>
-  <si>
-    <t>Vehicle exhaust</t>
-  </si>
-  <si>
-    <t>Petroleum solvents</t>
-  </si>
-  <si>
-    <t>Auto repair</t>
-  </si>
 </sst>
 </file>
 
@@ -205,9 +180,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -541,7 +515,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEA387BC-3A71-48D5-869C-430C29FEFC03}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2251DF4-E5D9-40AC-B472-BFFF46D6693B}">
   <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -579,28 +553,28 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>5.9914000000000002E-2</v>
+        <v>6.0009E-2</v>
       </c>
       <c r="C2">
-        <v>3.0085679836329201E-2</v>
+        <v>2.8591114056330299E-2</v>
       </c>
       <c r="D2">
-        <v>6.5163835208834495E-2</v>
+        <v>6.4781721327568598E-2</v>
       </c>
       <c r="E2">
-        <v>0.105364680722045</v>
+        <v>9.9716430605064701E-2</v>
       </c>
       <c r="F2">
-        <v>6.3378357887268102</v>
+        <v>6.6544094085693404</v>
       </c>
       <c r="G2">
-        <v>2.98202858439259</v>
+        <v>2.8534776760810998</v>
       </c>
       <c r="H2">
-        <v>6.11881658225058</v>
+        <v>6.3065816249313098</v>
       </c>
       <c r="I2">
-        <v>10.225519362189001</v>
+        <v>9.7157304722926892</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -608,28 +582,28 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.10259</v>
+        <v>0.10109</v>
       </c>
       <c r="C3">
-        <v>8.8281452678831099E-2</v>
+        <v>8.8979538035385497E-2</v>
       </c>
       <c r="D3">
-        <v>0.102764015978311</v>
+        <v>0.10303247098328901</v>
       </c>
       <c r="E3">
-        <v>0.119979968704855</v>
+        <v>0.120646840172729</v>
       </c>
       <c r="F3">
-        <v>26.8780918121338</v>
+        <v>27.146926879882798</v>
       </c>
       <c r="G3">
-        <v>22.836897959887299</v>
+        <v>23.190553909406201</v>
       </c>
       <c r="H3">
-        <v>26.649905869107702</v>
+        <v>26.935128475162799</v>
       </c>
       <c r="I3">
-        <v>30.640219536884601</v>
+        <v>31.3866946261934</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -637,28 +611,28 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1.0024E-2</v>
+        <v>1.0031999999999999E-2</v>
       </c>
       <c r="C4">
-        <v>5.8044090587837096E-3</v>
+        <v>5.5060517672674203E-3</v>
       </c>
       <c r="D4">
-        <v>1.0675965815070999E-2</v>
+        <v>1.07778083506855E-2</v>
       </c>
       <c r="E4">
-        <v>1.6753767235405798E-2</v>
+        <v>1.53417798327519E-2</v>
       </c>
       <c r="F4">
-        <v>7.0964469909668004</v>
+        <v>7.4299168586731001</v>
       </c>
       <c r="G4">
-        <v>3.6145113089699401</v>
+        <v>3.5964512652502698</v>
       </c>
       <c r="H4">
-        <v>6.7225962924969602</v>
+        <v>6.8814586270026297</v>
       </c>
       <c r="I4">
-        <v>10.8296921507607</v>
+        <v>9.98346170635795</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -666,28 +640,28 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>8.2553999999999995E-3</v>
+        <v>8.3081000000000006E-3</v>
       </c>
       <c r="C5">
-        <v>3.5553528016073598E-3</v>
+        <v>3.5700149410678298E-3</v>
       </c>
       <c r="D5">
-        <v>1.0067657353664401E-2</v>
+        <v>1.00807483345168E-2</v>
       </c>
       <c r="E5">
-        <v>2.0231156017584299E-2</v>
+        <v>1.7541083828521601E-2</v>
       </c>
       <c r="F5">
-        <v>4.41451120376587</v>
+        <v>4.6670660972595197</v>
       </c>
       <c r="G5">
-        <v>1.63461125185617</v>
+        <v>1.65480289348681</v>
       </c>
       <c r="H5">
-        <v>4.4363412915445499</v>
+        <v>4.5739719174529698</v>
       </c>
       <c r="I5">
-        <v>8.9413902241829604</v>
+        <v>7.9313853887283203</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -695,28 +669,28 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>8.3143999999999996E-2</v>
+        <v>8.2550999999999999E-2</v>
       </c>
       <c r="C6">
-        <v>6.1637479124644103E-2</v>
+        <v>6.3212472181955207E-2</v>
       </c>
       <c r="D6">
-        <v>8.5272886745902998E-2</v>
+        <v>8.5836726328624394E-2</v>
       </c>
       <c r="E6">
-        <v>0.112555139327722</v>
+        <v>0.106215026519801</v>
       </c>
       <c r="F6">
-        <v>14.769939422607401</v>
+        <v>15.160331726074199</v>
       </c>
       <c r="G6">
-        <v>10.042367251382201</v>
+        <v>10.420100032815901</v>
       </c>
       <c r="H6">
-        <v>14.307178176227</v>
+        <v>14.5232416009595</v>
       </c>
       <c r="I6">
-        <v>18.472862443942802</v>
+        <v>18.251797450084698</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -724,28 +698,28 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>2.7631000000000001E-3</v>
+        <v>2.6829000000000002E-3</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
       <c r="D7">
-        <v>3.1200218712455399E-3</v>
+        <v>2.9938025963688001E-3</v>
       </c>
       <c r="E7">
-        <v>7.3212759979345704E-3</v>
+        <v>7.1044736167689302E-3</v>
       </c>
       <c r="F7">
-        <v>8.3872318267822301</v>
+        <v>8.2636270523071307</v>
       </c>
       <c r="G7">
         <v>0</v>
       </c>
       <c r="H7">
-        <v>8.2382831610918306</v>
+        <v>8.0209027702786209</v>
       </c>
       <c r="I7">
-        <v>21.296637923625202</v>
+        <v>20.640659516847201</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
@@ -759,22 +733,22 @@
         <v>0</v>
       </c>
       <c r="D8">
-        <v>1.53788841415273E-3</v>
+        <v>1.53967702893864E-3</v>
       </c>
       <c r="E8">
-        <v>6.1608395423400197E-3</v>
+        <v>5.8431543872247398E-3</v>
       </c>
       <c r="F8">
-        <v>0.57956725358963002</v>
+        <v>0.68135815858840898</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8">
-        <v>1.5760677891938499</v>
+        <v>1.6998195335664901</v>
       </c>
       <c r="I8">
-        <v>6.8372867192847204</v>
+        <v>6.2141933728301604</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
@@ -785,25 +759,25 @@
         <v>0</v>
       </c>
       <c r="C9">
-        <v>2.7570829176765603E-20</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>6.9363923769712502E-4</v>
+        <v>6.9644282548109399E-4</v>
       </c>
       <c r="E9">
-        <v>2.3944429295602999E-3</v>
+        <v>2.2820844690569198E-3</v>
       </c>
       <c r="F9">
-        <v>0.68715125322341897</v>
+        <v>0.79414987564086903</v>
       </c>
       <c r="G9">
-        <v>5.9088167718135398E-17</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>1.54460621692158</v>
+        <v>1.5633488341480699</v>
       </c>
       <c r="I9">
-        <v>5.5407192232418696</v>
+        <v>5.3470298379964101</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -820,7 +794,7 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>4.4713868173292103E-3</v>
+        <v>4.4810929059171303E-3</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -832,7 +806,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>3.6437692489648401</v>
+        <v>3.6083658245853698</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -840,28 +814,28 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>2.6079000000000001E-2</v>
+        <v>2.598E-2</v>
       </c>
       <c r="C11">
-        <v>7.3708965772607297E-3</v>
+        <v>6.2171989315627299E-3</v>
       </c>
       <c r="D11">
-        <v>2.2598574907407101E-2</v>
+        <v>2.27614769011499E-2</v>
       </c>
       <c r="E11">
-        <v>3.7875315565784801E-2</v>
+        <v>3.7433803082254198E-2</v>
       </c>
       <c r="F11">
-        <v>9.0379447937011701</v>
+        <v>9.4095897674560494</v>
       </c>
       <c r="G11">
-        <v>2.2968056666551901</v>
+        <v>2.2660190681944501</v>
       </c>
       <c r="H11">
-        <v>7.89824928272688</v>
+        <v>7.8994552820219397</v>
       </c>
       <c r="I11">
-        <v>12.215066427048299</v>
+        <v>12.092946153550299</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -869,28 +843,28 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>5.2152999999999998E-2</v>
+        <v>5.1846000000000003E-2</v>
       </c>
       <c r="C12">
-        <v>2.1789305909201698E-2</v>
+        <v>2.6029541451587399E-2</v>
       </c>
       <c r="D12">
-        <v>5.0108881982289202E-2</v>
+        <v>5.0573651116851297E-2</v>
       </c>
       <c r="E12">
-        <v>6.6338243492123194E-2</v>
+        <v>6.5390166932360105E-2</v>
       </c>
       <c r="F12">
-        <v>11.8272867202759</v>
+        <v>12.2286033630371</v>
       </c>
       <c r="G12">
-        <v>4.9779157834499896</v>
+        <v>6.1211278257927102</v>
       </c>
       <c r="H12">
-        <v>11.1684024035038</v>
+        <v>11.459581892795899</v>
       </c>
       <c r="I12">
-        <v>14.7795926721478</v>
+        <v>15.020958106073699</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -898,28 +872,28 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>1.0496E-2</v>
+        <v>1.0324E-2</v>
       </c>
       <c r="C13">
-        <v>2.22929306549253E-3</v>
+        <v>3.6708177117255902E-3</v>
       </c>
       <c r="D13">
-        <v>1.0868979285585801E-2</v>
+        <v>1.09124866826029E-2</v>
       </c>
       <c r="E13">
-        <v>1.8316202434979001E-2</v>
+        <v>1.80836419372081E-2</v>
       </c>
       <c r="F13">
-        <v>15.095675468444799</v>
+        <v>15.229896545410201</v>
       </c>
       <c r="G13">
-        <v>2.56164050737129</v>
+        <v>4.3614841742890498</v>
       </c>
       <c r="H13">
-        <v>14.6594737068986</v>
+        <v>14.7652555933775</v>
       </c>
       <c r="I13">
-        <v>24.649147298714499</v>
+        <v>24.882980093759301</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -927,28 +901,28 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>1.1039999999999999E-2</v>
+        <v>1.0753E-2</v>
       </c>
       <c r="C14">
         <v>0</v>
       </c>
       <c r="D14">
-        <v>9.8008977823201802E-3</v>
+        <v>9.9432985372926597E-3</v>
       </c>
       <c r="E14">
-        <v>1.9123019454314098E-2</v>
+        <v>1.9418246351770901E-2</v>
       </c>
       <c r="F14">
-        <v>11.619752883911101</v>
+        <v>11.521076202392599</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
       <c r="H14">
-        <v>10.144829600845901</v>
+        <v>9.7606132136022907</v>
       </c>
       <c r="I14">
-        <v>19.3650134038602</v>
+        <v>19.768817771749301</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -956,28 +930,28 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>3.1035999999999998E-4</v>
+        <v>6.6969000000000002E-5</v>
       </c>
       <c r="C15">
         <v>0</v>
       </c>
       <c r="D15">
-        <v>2.31038824086562E-16</v>
+        <v>2.4958702639669099E-4</v>
       </c>
       <c r="E15">
-        <v>1.1961819799395401E-2</v>
+        <v>1.1943108366481501E-2</v>
       </c>
       <c r="F15">
-        <v>0.39173004031181302</v>
+        <v>3.86474368951895E-7</v>
       </c>
       <c r="G15">
         <v>0</v>
       </c>
       <c r="H15">
-        <v>1.99604590552567E-13</v>
+        <v>0.202106277242104</v>
       </c>
       <c r="I15">
-        <v>9.1670807626022892</v>
+        <v>8.8889761346740901</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -985,28 +959,28 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>6.9901E-3</v>
+        <v>6.7885000000000003E-3</v>
       </c>
       <c r="C16">
-        <v>4.7198979569377502E-3</v>
+        <v>4.8708374158302802E-3</v>
       </c>
       <c r="D16">
-        <v>7.40894573210243E-3</v>
+        <v>7.16345526718989E-3</v>
       </c>
       <c r="E16">
-        <v>1.0465115052122999E-2</v>
+        <v>1.0180742047877001E-2</v>
       </c>
       <c r="F16">
-        <v>5.8264951705932599</v>
+        <v>5.7211375236511204</v>
       </c>
       <c r="G16">
-        <v>4.0857993787415197</v>
+        <v>4.2661058095708499</v>
       </c>
       <c r="H16">
-        <v>6.2969350017226597</v>
+        <v>6.2381917632349104</v>
       </c>
       <c r="I16">
-        <v>9.0801132076475692</v>
+        <v>8.9684636677524505</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
@@ -1014,28 +988,28 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>2.138E-2</v>
+        <v>2.1191999999999999E-2</v>
       </c>
       <c r="C17">
-        <v>1.1164509547732701E-2</v>
+        <v>1.0883455196371201E-2</v>
       </c>
       <c r="D17">
-        <v>2.1015725576000999E-2</v>
+        <v>2.10006181371163E-2</v>
       </c>
       <c r="E17">
-        <v>2.87322129782791E-2</v>
+        <v>2.76919197884536E-2</v>
       </c>
       <c r="F17">
-        <v>7.7204122543334996</v>
+        <v>7.9332599639892596</v>
       </c>
       <c r="G17">
-        <v>4.0959583070135102</v>
+        <v>4.0056013054537596</v>
       </c>
       <c r="H17">
-        <v>7.6022279508014003</v>
+        <v>7.6993575025273797</v>
       </c>
       <c r="I17">
-        <v>10.136973762107001</v>
+        <v>10.112085587504099</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
@@ -1052,7 +1026,7 @@
         <v>0</v>
       </c>
       <c r="E18">
-        <v>6.1265690230345596E-3</v>
+        <v>5.45387459537185E-3</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -1064,7 +1038,7 @@
         <v>0</v>
       </c>
       <c r="I18">
-        <v>2.5589389338800101</v>
+        <v>2.3405140435924001</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
@@ -1072,28 +1046,28 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>5.0611000000000003E-2</v>
+        <v>4.9940999999999999E-2</v>
       </c>
       <c r="C19">
-        <v>3.4609367574746502E-2</v>
+        <v>3.4661676653846403E-2</v>
       </c>
       <c r="D19">
-        <v>4.9742056823589703E-2</v>
+        <v>4.9552127200790101E-2</v>
       </c>
       <c r="E19">
-        <v>6.3820624179022706E-2</v>
+        <v>6.1939924106256497E-2</v>
       </c>
       <c r="F19">
-        <v>8.0342226028442401</v>
+        <v>8.1723089218139595</v>
       </c>
       <c r="G19">
-        <v>5.7075464187541298</v>
+        <v>5.80607000254669</v>
       </c>
       <c r="H19">
-        <v>7.9534282108497401</v>
+        <v>8.0472622271795604</v>
       </c>
       <c r="I19">
-        <v>10.0009070275937</v>
+        <v>9.9306146698261095</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
@@ -1101,28 +1075,28 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>0.16492000000000001</v>
+        <v>0.16199</v>
       </c>
       <c r="C20">
-        <v>0.12908138953258</v>
+        <v>0.13270681873748999</v>
       </c>
       <c r="D20">
-        <v>0.16173440340055401</v>
+        <v>0.15960367996299801</v>
       </c>
       <c r="E20">
-        <v>0.182508636673617</v>
+        <v>0.17787873851757799</v>
       </c>
       <c r="F20">
-        <v>18.607387542724599</v>
+        <v>18.6877956390381</v>
       </c>
       <c r="G20">
-        <v>14.9655172407516</v>
+        <v>15.308112267673801</v>
       </c>
       <c r="H20">
-        <v>18.525587303494099</v>
+        <v>18.6238023704569</v>
       </c>
       <c r="I20">
-        <v>20.985096869248501</v>
+        <v>20.884783855904601</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
@@ -1130,28 +1104,28 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>0.35305999999999998</v>
+        <v>0.34759000000000001</v>
       </c>
       <c r="C21">
-        <v>0.27792671935497598</v>
+        <v>0.28429874550647699</v>
       </c>
       <c r="D21">
-        <v>0.34842121274961402</v>
+        <v>0.34449572723580801</v>
       </c>
       <c r="E21">
-        <v>0.39335270364101099</v>
+        <v>0.388056359582585</v>
       </c>
       <c r="F21">
-        <v>15.4435625076294</v>
+        <v>15.5905904769897</v>
       </c>
       <c r="G21">
-        <v>12.327920911126901</v>
+        <v>12.8854125200361</v>
       </c>
       <c r="H21">
-        <v>15.612613486626801</v>
+        <v>15.688310396336901</v>
       </c>
       <c r="I21">
-        <v>17.757182105501599</v>
+        <v>17.7594239356843</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
@@ -1159,28 +1133,28 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>4.7916E-2</v>
+        <v>4.6911000000000001E-2</v>
       </c>
       <c r="C22">
-        <v>3.3030944901364101E-2</v>
+        <v>3.2976784537940097E-2</v>
       </c>
       <c r="D22">
-        <v>4.7291898026557602E-2</v>
+        <v>4.7104377239262897E-2</v>
       </c>
       <c r="E22">
-        <v>7.3893466768013102E-2</v>
+        <v>7.0760720319373305E-2</v>
       </c>
       <c r="F22">
-        <v>31.696756362915</v>
+        <v>31.530969619751001</v>
       </c>
       <c r="G22">
-        <v>26.324669337343899</v>
+        <v>26.154328943673001</v>
       </c>
       <c r="H22">
-        <v>36.512282345307803</v>
+        <v>36.120235952381798</v>
       </c>
       <c r="I22">
-        <v>52.978246220889297</v>
+        <v>50.896434235944703</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
@@ -1188,28 +1162,28 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>2.9871999999999999E-2</v>
+        <v>2.8552999999999999E-2</v>
       </c>
       <c r="C23">
-        <v>1.5321285343932199E-2</v>
+        <v>1.52536740367154E-2</v>
       </c>
       <c r="D23">
-        <v>3.3271920541309098E-2</v>
+        <v>3.2788554910596603E-2</v>
       </c>
       <c r="E23">
-        <v>5.5275098469870498E-2</v>
+        <v>5.4812381875976403E-2</v>
       </c>
       <c r="F23">
-        <v>4.1782760620117196</v>
+        <v>3.9410359859466602</v>
       </c>
       <c r="G23">
-        <v>2.31411670437353</v>
+        <v>2.4317924048019499</v>
       </c>
       <c r="H23">
-        <v>5.0617393226599301</v>
+        <v>5.0866115952900701</v>
       </c>
       <c r="I23">
-        <v>8.41677170763659</v>
+        <v>8.4905662116620704</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
@@ -1217,28 +1191,28 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>2.9554E-3</v>
+        <v>2.9272999999999999E-3</v>
       </c>
       <c r="C24">
-        <v>9.1857438179140504E-4</v>
+        <v>1.0462575430117899E-3</v>
       </c>
       <c r="D24">
-        <v>2.8886054991950601E-3</v>
+        <v>2.9157916328005498E-3</v>
       </c>
       <c r="E24">
-        <v>4.3611126496853597E-3</v>
+        <v>4.4534994569480199E-3</v>
       </c>
       <c r="F24">
-        <v>19.233907699585</v>
+        <v>19.595653533935501</v>
       </c>
       <c r="G24">
-        <v>5.17683910323208</v>
+        <v>5.69554286495553</v>
       </c>
       <c r="H24">
-        <v>18.346488686564498</v>
+        <v>18.8951441872758</v>
       </c>
       <c r="I24">
-        <v>30.7371221181184</v>
+        <v>31.4054013570519</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
@@ -1246,28 +1220,28 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>0.13422000000000001</v>
+        <v>0.13161</v>
       </c>
       <c r="C25">
-        <v>9.5477132322245695E-2</v>
+        <v>9.5356191772430099E-2</v>
       </c>
       <c r="D25">
-        <v>0.134634067064861</v>
+        <v>0.13392247308757901</v>
       </c>
       <c r="E25">
-        <v>0.19008280010923301</v>
+        <v>0.191543494431448</v>
       </c>
       <c r="F25">
-        <v>49.871173858642599</v>
+        <v>49.817413330078097</v>
       </c>
       <c r="G25">
-        <v>38.334263239518997</v>
+        <v>38.499489618549397</v>
       </c>
       <c r="H25">
-        <v>51.0157033852579</v>
+        <v>50.943572146574503</v>
       </c>
       <c r="I25">
-        <v>62.875175441412601</v>
+        <v>63.564636118868599</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
@@ -1284,7 +1258,7 @@
         <v>0</v>
       </c>
       <c r="E26">
-        <v>1.1031680788509701E-3</v>
+        <v>8.7537648600012196E-4</v>
       </c>
       <c r="F26">
         <v>0</v>
@@ -1296,7 +1270,7 @@
         <v>0</v>
       </c>
       <c r="I26">
-        <v>5.1674462401045096</v>
+        <v>4.31550051879361</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
@@ -1304,28 +1278,28 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>0.10095</v>
+        <v>9.9085000000000006E-2</v>
       </c>
       <c r="C27">
-        <v>7.8044064603199306E-2</v>
+        <v>7.9166387849622197E-2</v>
       </c>
       <c r="D27">
-        <v>0.100668930239926</v>
+        <v>0.10131211245822801</v>
       </c>
       <c r="E27">
-        <v>0.131738800635087</v>
+        <v>0.13568086891811099</v>
       </c>
       <c r="F27">
-        <v>85.501449584960895</v>
+        <v>85.532447814941406</v>
       </c>
       <c r="G27">
-        <v>70.326015310402695</v>
+        <v>71.356740586302095</v>
       </c>
       <c r="H27">
-        <v>82.8704245129193</v>
+        <v>82.438706906404505</v>
       </c>
       <c r="I27">
-        <v>88.553096504132398</v>
+        <v>89.342649827489296</v>
       </c>
     </row>
   </sheetData>
@@ -1334,7 +1308,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A44BFF1A-7865-44AF-96A7-B311A6D8F610}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8702E11-6E04-403A-AE95-0D01F6A4C1B5}">
   <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -1372,28 +1346,28 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.23862</v>
+        <v>4.6098E-2</v>
       </c>
       <c r="C2">
-        <v>0.19923074887219699</v>
+        <v>3.7056731293550998E-2</v>
       </c>
       <c r="D2">
-        <v>0.23000743266774901</v>
+        <v>6.0071216548635502E-2</v>
       </c>
       <c r="E2">
-        <v>0.25726824872839499</v>
+        <v>8.9610423482023402E-2</v>
       </c>
       <c r="F2">
-        <v>22.392499923706101</v>
+        <v>4.7604432106018102</v>
       </c>
       <c r="G2">
-        <v>18.328492372119499</v>
+        <v>3.4728564980588499</v>
       </c>
       <c r="H2">
-        <v>21.883938461369802</v>
+        <v>5.8155920055156098</v>
       </c>
       <c r="I2">
-        <v>25.1030790592946</v>
+        <v>8.8306993256677409</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -1401,28 +1375,28 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>6.3564999999999997E-2</v>
+        <v>4.8344999999999999E-2</v>
       </c>
       <c r="C3">
-        <v>4.3985868565007899E-2</v>
+        <v>2.2445308690556099E-2</v>
       </c>
       <c r="D3">
-        <v>6.65494883177562E-2</v>
+        <v>4.5028126831738201E-2</v>
       </c>
       <c r="E3">
-        <v>8.9441157352346701E-2</v>
+        <v>6.3545018369818698E-2</v>
       </c>
       <c r="F3">
-        <v>16.488561630248999</v>
+        <v>13.128002166748001</v>
       </c>
       <c r="G3">
-        <v>11.341462365875801</v>
+        <v>5.72737807627969</v>
       </c>
       <c r="H3">
-        <v>17.415862708762699</v>
+        <v>11.837575724802001</v>
       </c>
       <c r="I3">
-        <v>23.3462334225141</v>
+        <v>17.3585150584837</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -1430,28 +1404,28 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>4.1124000000000001E-2</v>
+        <v>3.8758E-3</v>
       </c>
       <c r="C4">
-        <v>3.2513419146841402E-2</v>
+        <v>3.97417565821322E-3</v>
       </c>
       <c r="D4">
-        <v>3.8637410845736103E-2</v>
+        <v>7.0386495187532601E-3</v>
       </c>
       <c r="E4">
-        <v>4.36382254033955E-2</v>
+        <v>1.13746212463827E-2</v>
       </c>
       <c r="F4">
-        <v>25.605007171630898</v>
+        <v>2.79656887054443</v>
       </c>
       <c r="G4">
-        <v>20.303543677617899</v>
+        <v>2.51157377344459</v>
       </c>
       <c r="H4">
-        <v>24.383286472921601</v>
+        <v>4.5459589124333801</v>
       </c>
       <c r="I4">
-        <v>28.276902032154599</v>
+        <v>7.5660550966109401</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -1459,28 +1433,28 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>7.2364999999999999E-2</v>
+        <v>6.9702000000000002E-3</v>
       </c>
       <c r="C5">
-        <v>5.6823074419336601E-2</v>
+        <v>5.7035139601573298E-3</v>
       </c>
       <c r="D5">
-        <v>6.5949638259263296E-2</v>
+        <v>9.8965626657277692E-3</v>
       </c>
       <c r="E5">
-        <v>7.3686953257249693E-2</v>
+        <v>1.7548779752387798E-2</v>
       </c>
       <c r="F5">
-        <v>31.0026969909668</v>
+        <v>3.3937420845031698</v>
       </c>
       <c r="G5">
-        <v>24.8976145715217</v>
+        <v>2.5132058505366501</v>
       </c>
       <c r="H5">
-        <v>29.304837354906599</v>
+        <v>4.4590315828335703</v>
       </c>
       <c r="I5">
-        <v>32.408133521166498</v>
+        <v>8.0567019067135206</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -1488,28 +1462,28 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>0.15074000000000001</v>
+        <v>7.0136000000000004E-2</v>
       </c>
       <c r="C6">
-        <v>8.6406230798133504E-2</v>
+        <v>4.0768137925705002E-2</v>
       </c>
       <c r="D6">
-        <v>0.14755723617441599</v>
+        <v>6.8769956199202495E-2</v>
       </c>
       <c r="E6">
-        <v>0.190551243384006</v>
+        <v>0.100267596553759</v>
       </c>
       <c r="F6">
-        <v>24.710771560668899</v>
+        <v>11.482795715331999</v>
       </c>
       <c r="G6">
-        <v>13.767316505652699</v>
+        <v>6.9079997980663599</v>
       </c>
       <c r="H6">
-        <v>25.335023239064402</v>
+        <v>11.398326851023899</v>
       </c>
       <c r="I6">
-        <v>33.306573295901998</v>
+        <v>16.555345860553299</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -1517,28 +1491,28 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>2.0836E-2</v>
+        <v>4.8025000000000003E-3</v>
       </c>
       <c r="C7">
-        <v>1.29249615113697E-2</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>1.8067530556903699E-2</v>
+        <v>2.98589543384689E-3</v>
       </c>
       <c r="E7">
-        <v>2.3503675280447299E-2</v>
+        <v>8.6276870071099396E-3</v>
       </c>
       <c r="F7">
-        <v>50.957592010497997</v>
+        <v>12.9571418762207</v>
       </c>
       <c r="G7">
-        <v>31.9343571128205</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>48.112768878400303</v>
+        <v>8.6135209962353194</v>
       </c>
       <c r="I7">
-        <v>62.074550261816903</v>
+        <v>24.635740572760501</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
@@ -1546,28 +1520,28 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>3.6735999999999998E-2</v>
+        <v>0</v>
       </c>
       <c r="C8">
-        <v>2.4941430044708199E-2</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>3.2904295927417102E-2</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>4.1757656107760999E-2</v>
+        <v>2.7591639213160601E-3</v>
       </c>
       <c r="F8">
-        <v>37.562232971191399</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>26.444172068664201</v>
+        <v>0</v>
       </c>
       <c r="H8">
-        <v>34.902787724804298</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <v>42.729871354058901</v>
+        <v>3.07093388609659</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
@@ -1575,28 +1549,28 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>1.4619999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="C9">
-        <v>1.00238406700508E-2</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>1.32840204060317E-2</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>1.67396618873321E-2</v>
+        <v>1.22642018216733E-3</v>
       </c>
       <c r="F9">
-        <v>31.9096565246582</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>22.4774216699658</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>29.704130734333699</v>
+        <v>0</v>
       </c>
       <c r="I9">
-        <v>37.952599970500799</v>
+        <v>2.9388195501157801</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -1604,28 +1578,28 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>4.3232E-2</v>
+        <v>0</v>
       </c>
       <c r="C10">
-        <v>2.7399114376980199E-2</v>
+        <v>0</v>
       </c>
       <c r="D10">
-        <v>3.8133996846076802E-2</v>
+        <v>1.3090829000064899E-3</v>
       </c>
       <c r="E10">
-        <v>5.0186326704101197E-2</v>
+        <v>7.4553985933742198E-3</v>
       </c>
       <c r="F10">
-        <v>34.601303100585902</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>21.631160420117499</v>
+        <v>0</v>
       </c>
       <c r="H10">
-        <v>31.138982252300099</v>
+        <v>1.0977260320203399</v>
       </c>
       <c r="I10">
-        <v>41.321190938729103</v>
+        <v>6.1463239374584102</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -1633,28 +1607,28 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>8.6376000000000005E-3</v>
+        <v>0</v>
       </c>
       <c r="C11">
         <v>0</v>
       </c>
       <c r="D11">
-        <v>1.17039325053687E-2</v>
+        <v>1.1504919562477E-2</v>
       </c>
       <c r="E11">
-        <v>4.8145479373126597E-2</v>
+        <v>3.73600606892713E-2</v>
       </c>
       <c r="F11">
-        <v>3.3940303325653098</v>
+        <v>0</v>
       </c>
       <c r="G11">
         <v>0</v>
       </c>
       <c r="H11">
-        <v>3.99952372008921</v>
+        <v>4.0715303523122204</v>
       </c>
       <c r="I11">
-        <v>17.6586262056774</v>
+        <v>12.285680597451501</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -1662,28 +1636,28 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>1.0113E-2</v>
       </c>
       <c r="C12">
         <v>0</v>
       </c>
       <c r="D12">
-        <v>5.9364295048110097E-18</v>
+        <v>2.4104641123710101E-2</v>
       </c>
       <c r="E12">
-        <v>3.2964570744158803E-2</v>
+        <v>4.3022136292177E-2</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>3.32449579238892</v>
       </c>
       <c r="G12">
         <v>0</v>
       </c>
       <c r="H12">
-        <v>1.2550274952594E-15</v>
+        <v>5.6027735738662203</v>
       </c>
       <c r="I12">
-        <v>7.1046349403157798</v>
+        <v>9.6418786625357207</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -1691,28 +1665,28 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>3.8455999999999997E-2</v>
+        <v>7.9596000000000007E-3</v>
       </c>
       <c r="C13">
-        <v>2.3062200434388499E-2</v>
+        <v>5.7548365707214898E-4</v>
       </c>
       <c r="D13">
-        <v>3.51608685584038E-2</v>
+        <v>6.7669531072989701E-3</v>
       </c>
       <c r="E13">
-        <v>4.8586698378932799E-2</v>
+        <v>1.7492789258011201E-2</v>
       </c>
       <c r="F13">
-        <v>48.7621040344238</v>
+        <v>10.2966651916504</v>
       </c>
       <c r="G13">
-        <v>32.0502057914265</v>
+        <v>0.71581986790665297</v>
       </c>
       <c r="H13">
-        <v>46.7640470293397</v>
+        <v>9.14451104173129</v>
       </c>
       <c r="I13">
-        <v>61.077968164009398</v>
+        <v>24.482191887602401</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -1720,28 +1694,28 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>5.7182999999999998E-2</v>
+        <v>7.4454999999999996E-4</v>
       </c>
       <c r="C14">
-        <v>2.8162841651337801E-2</v>
+        <v>0</v>
       </c>
       <c r="D14">
-        <v>4.8077287599500501E-2</v>
+        <v>5.6237700238723697E-4</v>
       </c>
       <c r="E14">
-        <v>7.2293720289849997E-2</v>
+        <v>1.7915798715288499E-2</v>
       </c>
       <c r="F14">
-        <v>51.631767272949197</v>
+        <v>1.46115839481354</v>
       </c>
       <c r="G14">
-        <v>29.236108020187899</v>
+        <v>0</v>
       </c>
       <c r="H14">
-        <v>46.160239009525696</v>
+        <v>0.562825285116626</v>
       </c>
       <c r="I14">
-        <v>60.188900789978099</v>
+        <v>16.533885778781102</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -1749,28 +1723,28 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>4.5706999999999998E-2</v>
+        <v>9.8597000000000008E-3</v>
       </c>
       <c r="C15">
-        <v>2.0227849352257101E-2</v>
+        <v>0</v>
       </c>
       <c r="D15">
-        <v>3.9536192409444802E-2</v>
+        <v>6.3500024831008098E-3</v>
       </c>
       <c r="E15">
-        <v>5.6827968110290797E-2</v>
+        <v>2.2594663041679602E-2</v>
       </c>
       <c r="F15">
-        <v>33.223064422607401</v>
+        <v>8.3268566131591797</v>
       </c>
       <c r="G15">
-        <v>15.204015752616</v>
+        <v>0</v>
       </c>
       <c r="H15">
-        <v>30.1992740554245</v>
+        <v>4.9509313065008902</v>
       </c>
       <c r="I15">
-        <v>42.934868005175503</v>
+        <v>18.3996577815645</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -1778,28 +1752,28 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>2.3082999999999999E-2</v>
+        <v>9.3991999999999999E-3</v>
       </c>
       <c r="C16">
-        <v>1.51650119692694E-2</v>
+        <v>4.5791048647724503E-3</v>
       </c>
       <c r="D16">
-        <v>2.1751312152668401E-2</v>
+        <v>7.9066383857362092E-3</v>
       </c>
       <c r="E16">
-        <v>2.74085608219038E-2</v>
+        <v>1.2931099977117499E-2</v>
       </c>
       <c r="F16">
-        <v>19.2623291015625</v>
+        <v>8.3912172317504901</v>
       </c>
       <c r="G16">
-        <v>12.795771696230601</v>
+        <v>4.0552297365288696</v>
       </c>
       <c r="H16">
-        <v>18.520432025564102</v>
+        <v>6.8999802721785803</v>
       </c>
       <c r="I16">
-        <v>23.841652684311999</v>
+        <v>11.070863493923399</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
@@ -1807,28 +1781,28 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>1.5500999999999999E-2</v>
+        <v>1.1773E-2</v>
       </c>
       <c r="C17">
-        <v>1.0545818307252699E-2</v>
+        <v>7.2792075159856503E-3</v>
       </c>
       <c r="D17">
-        <v>1.7955246391384998E-2</v>
+        <v>1.70989995271086E-2</v>
       </c>
       <c r="E17">
-        <v>2.6893383602762101E-2</v>
+        <v>2.4113128852232601E-2</v>
       </c>
       <c r="F17">
-        <v>6.0578355789184597</v>
+        <v>4.8983464241027797</v>
       </c>
       <c r="G17">
-        <v>3.7620460878895301</v>
+        <v>2.7184999852707601</v>
       </c>
       <c r="H17">
-        <v>6.4800687070939</v>
+        <v>6.22937991225945</v>
       </c>
       <c r="I17">
-        <v>9.9431606779298392</v>
+        <v>8.6938362482116194</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
@@ -1836,28 +1810,28 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>4.1815999999999999E-2</v>
+        <v>0</v>
       </c>
       <c r="C18">
-        <v>2.1214027992718199E-2</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>3.7527798861675801E-2</v>
+        <v>2.0318325167756001E-3</v>
       </c>
       <c r="E18">
-        <v>5.8247880463440198E-2</v>
+        <v>1.3839549740233201E-2</v>
       </c>
       <c r="F18">
-        <v>17.7256774902344</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>8.3495803964195403</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>15.5830459105859</v>
+        <v>0.83587192800436705</v>
       </c>
       <c r="I18">
-        <v>25.313084149872299</v>
+        <v>5.8026836416042498</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
@@ -1865,28 +1839,28 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>4.6421999999999998E-2</v>
+        <v>2.6986E-2</v>
       </c>
       <c r="C19">
-        <v>3.1518134826476002E-2</v>
+        <v>1.9088537701919501E-2</v>
       </c>
       <c r="D19">
-        <v>4.9138126153445802E-2</v>
+        <v>3.6152014711299599E-2</v>
       </c>
       <c r="E19">
-        <v>6.7023736043661603E-2</v>
+        <v>5.5659096815553102E-2</v>
       </c>
       <c r="F19">
-        <v>7.8335323333740199</v>
+        <v>4.9851183891296396</v>
       </c>
       <c r="G19">
-        <v>4.9100412065383301</v>
+        <v>3.12619521335106</v>
       </c>
       <c r="H19">
-        <v>7.7777260451377499</v>
+        <v>5.8446249391235403</v>
       </c>
       <c r="I19">
-        <v>11.0399576204574</v>
+        <v>8.8730080727693004</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
@@ -1894,28 +1868,28 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>3.1489000000000003E-2</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>1.2322144009140799E-2</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>4.9190782955084798E-2</v>
       </c>
       <c r="E20">
-        <v>3.4530745222643801E-2</v>
+        <v>7.2261660727117094E-2</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>5.0394935607910201</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>1.26866687852185</v>
       </c>
       <c r="H20">
-        <v>0</v>
+        <v>5.7659073125529696</v>
       </c>
       <c r="I20">
-        <v>3.9313853271415802</v>
+        <v>8.4213491327551893</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
@@ -1923,28 +1897,28 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>4.0396000000000001E-2</v>
+        <v>0.19442000000000001</v>
       </c>
       <c r="C21">
-        <v>2.34185445144349E-2</v>
+        <v>8.8903501450994807E-2</v>
       </c>
       <c r="D21">
-        <v>8.0402161531065497E-2</v>
+        <v>0.19587224409131601</v>
       </c>
       <c r="E21">
-        <v>0.169972964288751</v>
+        <v>0.23351747504588199</v>
       </c>
       <c r="F21">
-        <v>2.3239233493804901</v>
+        <v>9.6271505355834996</v>
       </c>
       <c r="G21">
-        <v>1.04439150762647</v>
+        <v>4.10587837366774</v>
       </c>
       <c r="H21">
-        <v>3.6183772595110901</v>
+        <v>8.8717316335561893</v>
       </c>
       <c r="I21">
-        <v>7.8136830774569503</v>
+        <v>10.656777994219301</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
@@ -1952,28 +1926,28 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>6.3893000000000005E-2</v>
       </c>
       <c r="C22">
         <v>0</v>
       </c>
       <c r="D22">
-        <v>5.6681744720819805E-4</v>
+        <v>4.4425761272652201E-2</v>
       </c>
       <c r="E22">
-        <v>5.46345374581267E-2</v>
+        <v>6.8260508375967199E-2</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>46.1369018554688</v>
       </c>
       <c r="G22">
         <v>0</v>
       </c>
       <c r="H22">
-        <v>0.37665989041029402</v>
+        <v>34.486869984626402</v>
       </c>
       <c r="I22">
-        <v>51.650977740666796</v>
+        <v>47.2373154223434</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
@@ -1981,28 +1955,28 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>0.12135</v>
+        <v>1.0465E-2</v>
       </c>
       <c r="C23">
-        <v>4.5852509805626003E-2</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>0.101473624103224</v>
+        <v>1.16820301079942E-2</v>
       </c>
       <c r="E23">
-        <v>0.16707613955470699</v>
+        <v>5.4957877941618799E-2</v>
       </c>
       <c r="F23">
-        <v>18.153072357177699</v>
+        <v>2.4195442199707</v>
       </c>
       <c r="G23">
-        <v>6.8336268304483099</v>
+        <v>0</v>
       </c>
       <c r="H23">
-        <v>15.513510780388</v>
+        <v>1.8484472523457001</v>
       </c>
       <c r="I23">
-        <v>25.711972265414701</v>
+        <v>8.6878279400336496</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
@@ -2010,28 +1984,28 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>2.7501000000000001E-3</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>6.9852911272788305E-4</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>2.6681466104504E-3</v>
       </c>
       <c r="E24">
-        <v>1.7509649172291E-3</v>
+        <v>4.4226029337382797E-3</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>19.890163421630898</v>
       </c>
       <c r="G24">
-        <v>0</v>
+        <v>4.0442783750653204</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>17.476145296063301</v>
       </c>
       <c r="I24">
-        <v>11.2956401748104</v>
+        <v>28.012316194691898</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
@@ -2039,28 +2013,28 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>0.12015000000000001</v>
+        <v>1.9806000000000001E-2</v>
       </c>
       <c r="C25">
-        <v>7.1172699236286302E-2</v>
+        <v>0</v>
       </c>
       <c r="D25">
-        <v>0.103908616891734</v>
+        <v>1.2927392062846601E-2</v>
       </c>
       <c r="E25">
-        <v>0.13707007398249901</v>
+        <v>6.6348144743014995E-2</v>
       </c>
       <c r="F25">
-        <v>42.370845794677699</v>
+        <v>7.6983475685119602</v>
       </c>
       <c r="G25">
-        <v>25.000647029701401</v>
+        <v>0</v>
       </c>
       <c r="H25">
-        <v>39.808277945297597</v>
+        <v>4.7756200757829799</v>
       </c>
       <c r="I25">
-        <v>52.078815358123002</v>
+        <v>23.3756067797285</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
@@ -2068,28 +2042,28 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>1.7052999999999999E-2</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>7.3136715342637503E-3</v>
       </c>
       <c r="D26">
-        <v>8.5325333139903104E-4</v>
+        <v>1.1735847779829899E-2</v>
       </c>
       <c r="E26">
-        <v>4.6226349302260199E-3</v>
+        <v>2.0767636557051199E-2</v>
       </c>
       <c r="F26">
-        <v>3.5155055522918701</v>
+        <v>83.725570678710895</v>
       </c>
       <c r="G26">
-        <v>0</v>
+        <v>59.862452043833301</v>
       </c>
       <c r="H26">
-        <v>5.13139480179579</v>
+        <v>73.420799620691398</v>
       </c>
       <c r="I26">
-        <v>33.126316643305799</v>
+        <v>87.837890326746901</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
@@ -2097,28 +2071,28 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>5.4930999999999999E-3</v>
+        <v>0</v>
       </c>
       <c r="C27">
         <v>0</v>
       </c>
       <c r="D27">
-        <v>5.4306858540227303E-3</v>
+        <v>0</v>
       </c>
       <c r="E27">
-        <v>2.0863121413000101E-2</v>
+        <v>1.53723383227687E-2</v>
       </c>
       <c r="F27">
-        <v>5.4487714767456099</v>
+        <v>0</v>
       </c>
       <c r="G27">
         <v>0</v>
       </c>
       <c r="H27">
-        <v>4.6119067571806101</v>
+        <v>0</v>
       </c>
       <c r="I27">
-        <v>16.476872840933002</v>
+        <v>11.9624696580765</v>
       </c>
     </row>
   </sheetData>
@@ -2127,7 +2101,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72C8D7E8-0421-450F-B044-9715EBC6D5D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD9A6C4F-6BEF-4A29-9849-7BE4D83C5F21}">
   <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -2165,28 +2139,28 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.53474999999999995</v>
+        <v>0.52612999999999999</v>
       </c>
       <c r="C2">
-        <v>0.42933298080019699</v>
+        <v>0.40641397737849599</v>
       </c>
       <c r="D2">
-        <v>0.52964168723258798</v>
+        <v>0.517657161024488</v>
       </c>
       <c r="E2">
-        <v>0.63368881580528003</v>
+        <v>0.61321254676779602</v>
       </c>
       <c r="F2">
-        <v>51.067081451416001</v>
+        <v>50.799365997314503</v>
       </c>
       <c r="G2">
-        <v>42.576827308188903</v>
+        <v>40.9204745394361</v>
       </c>
       <c r="H2">
-        <v>50.9685326016332</v>
+        <v>50.4348793862668</v>
       </c>
       <c r="I2">
-        <v>56.705251490942203</v>
+        <v>56.6067715297565</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -2194,28 +2168,28 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.15819</v>
+        <v>0.15548000000000001</v>
       </c>
       <c r="C3">
-        <v>0.113179217658625</v>
+        <v>0.11385941972896101</v>
       </c>
       <c r="D3">
-        <v>0.153372522607297</v>
+        <v>0.15030891687336501</v>
       </c>
       <c r="E3">
-        <v>0.201499126202006</v>
+        <v>0.19489202820450899</v>
       </c>
       <c r="F3">
-        <v>39.277618408203097</v>
+        <v>39.066944122314503</v>
       </c>
       <c r="G3">
-        <v>32.392205391429997</v>
+        <v>31.925788909301399</v>
       </c>
       <c r="H3">
-        <v>39.363796428537697</v>
+        <v>39.122508034931698</v>
       </c>
       <c r="I3">
-        <v>47.804093446321602</v>
+        <v>47.094110615308402</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -2223,28 +2197,28 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>8.0782000000000007E-2</v>
+        <v>7.9477999999999993E-2</v>
       </c>
       <c r="C4">
-        <v>6.6522850598816102E-2</v>
+        <v>6.21337161481696E-2</v>
       </c>
       <c r="D4">
-        <v>8.0091451281372003E-2</v>
+        <v>7.8328925704363395E-2</v>
       </c>
       <c r="E4">
-        <v>9.5423270674538402E-2</v>
+        <v>9.2201112226479101E-2</v>
       </c>
       <c r="F4">
-        <v>51.3899116516113</v>
+        <v>51.120426177978501</v>
       </c>
       <c r="G4">
-        <v>44.079809350376301</v>
+        <v>43.141597412354599</v>
       </c>
       <c r="H4">
-        <v>51.159818191036202</v>
+        <v>50.691381132314199</v>
       </c>
       <c r="I4">
-        <v>57.015831959173298</v>
+        <v>56.753835927118203</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -2252,28 +2226,28 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0.10209</v>
+        <v>0.10047</v>
       </c>
       <c r="C5">
-        <v>7.8164888118019901E-2</v>
+        <v>7.3308820696674604E-2</v>
       </c>
       <c r="D5">
-        <v>0.10251415206018701</v>
+        <v>0.10074632806572301</v>
       </c>
       <c r="E5">
-        <v>0.12742765718242999</v>
+        <v>0.123748630466403</v>
       </c>
       <c r="F5">
-        <v>44.976047515869098</v>
+        <v>44.751953125</v>
       </c>
       <c r="G5">
-        <v>35.7577047329412</v>
+        <v>35.391900479517297</v>
       </c>
       <c r="H5">
-        <v>45.771677370595498</v>
+        <v>45.240518769932102</v>
       </c>
       <c r="I5">
-        <v>53.360563723286099</v>
+        <v>52.378333919567503</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -2281,28 +2255,28 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>0.30134</v>
+        <v>0.29676000000000002</v>
       </c>
       <c r="C6">
-        <v>0.22342681366567099</v>
+        <v>0.21737895304090299</v>
       </c>
       <c r="D6">
-        <v>0.289750979272826</v>
+        <v>0.28591490382436202</v>
       </c>
       <c r="E6">
-        <v>0.37284412536544997</v>
+        <v>0.36035291493354199</v>
       </c>
       <c r="F6">
-        <v>48.836593627929702</v>
+        <v>48.606575012207003</v>
       </c>
       <c r="G6">
-        <v>40.1880471742897</v>
+        <v>39.747959938959603</v>
       </c>
       <c r="H6">
-        <v>48.519311933756299</v>
+        <v>48.776804909425302</v>
       </c>
       <c r="I6">
-        <v>57.329298173113202</v>
+        <v>56.0452267425744</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -2310,28 +2284,28 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>3.483E-3</v>
+        <v>3.4312000000000001E-3</v>
       </c>
       <c r="C7">
-        <v>9.1507935779985502E-4</v>
+        <v>1.0213605696704599E-3</v>
       </c>
       <c r="D7">
-        <v>3.8629072419522899E-3</v>
+        <v>3.6127003022768502E-3</v>
       </c>
       <c r="E7">
-        <v>2.07833159986082E-2</v>
+        <v>1.8910539167193E-2</v>
       </c>
       <c r="F7">
-        <v>8.3708858489990199</v>
+        <v>8.3834161758422905</v>
       </c>
       <c r="G7">
-        <v>2.9657127215146999</v>
+        <v>3.4051640312060898</v>
       </c>
       <c r="H7">
-        <v>10.0428279190777</v>
+        <v>9.6617421675875406</v>
       </c>
       <c r="I7">
-        <v>42.9836412047351</v>
+        <v>39.888905154701902</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
@@ -2339,28 +2313,28 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>3.3964000000000001E-2</v>
+        <v>3.3411999999999997E-2</v>
       </c>
       <c r="C8">
-        <v>2.41461054280485E-2</v>
+        <v>2.3595838732932601E-2</v>
       </c>
       <c r="D8">
-        <v>3.5822223113230599E-2</v>
+        <v>3.49332861327077E-2</v>
       </c>
       <c r="E8">
-        <v>4.8263848902524498E-2</v>
+        <v>4.61302003986679E-2</v>
       </c>
       <c r="F8">
-        <v>36.104515075683601</v>
+        <v>35.905120849609403</v>
       </c>
       <c r="G8">
-        <v>26.601962170031801</v>
+        <v>27.159589204443499</v>
       </c>
       <c r="H8">
-        <v>37.581187426246899</v>
+        <v>37.048458310312398</v>
       </c>
       <c r="I8">
-        <v>48.402589295194403</v>
+        <v>47.240957960399399</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
@@ -2368,28 +2342,28 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>1.6808E-2</v>
+        <v>1.6531000000000001E-2</v>
       </c>
       <c r="C9">
-        <v>1.2363427996626101E-2</v>
+        <v>1.2283170969451199E-2</v>
       </c>
       <c r="D9">
-        <v>1.75937932121699E-2</v>
+        <v>1.7040459402961099E-2</v>
       </c>
       <c r="E9">
-        <v>2.4072369668504699E-2</v>
+        <v>2.2891154614998299E-2</v>
       </c>
       <c r="F9">
-        <v>38.101814270019503</v>
+        <v>37.891124725341797</v>
       </c>
       <c r="G9">
-        <v>30.396706769140899</v>
+        <v>30.183895510567901</v>
       </c>
       <c r="H9">
-        <v>39.3064781651251</v>
+        <v>38.875022870248301</v>
       </c>
       <c r="I9">
-        <v>49.731647468164503</v>
+        <v>48.447051724284101</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -2397,28 +2371,28 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>3.4936000000000002E-2</v>
+        <v>3.4368000000000003E-2</v>
       </c>
       <c r="C10">
-        <v>2.4206148875927602E-2</v>
+        <v>2.27446793182472E-2</v>
       </c>
       <c r="D10">
-        <v>3.82128280071641E-2</v>
+        <v>3.63003919053849E-2</v>
       </c>
       <c r="E10">
-        <v>5.9128178199987599E-2</v>
+        <v>5.5190255443207499E-2</v>
       </c>
       <c r="F10">
-        <v>29.638240814208999</v>
+        <v>29.5076293945313</v>
       </c>
       <c r="G10">
-        <v>21.301259770543499</v>
+        <v>20.840980436853499</v>
       </c>
       <c r="H10">
-        <v>30.965547157090601</v>
+        <v>30.623531079341301</v>
       </c>
       <c r="I10">
-        <v>44.5563576497659</v>
+        <v>42.6259136098518</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -2426,28 +2400,28 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>0.18421999999999999</v>
+        <v>0.18104999999999999</v>
       </c>
       <c r="C11">
-        <v>0.12661391203248501</v>
+        <v>0.124569320316195</v>
       </c>
       <c r="D11">
-        <v>0.17512583912486701</v>
+        <v>0.168460569357783</v>
       </c>
       <c r="E11">
-        <v>0.20401372020960901</v>
+        <v>0.19863535106829699</v>
       </c>
       <c r="F11">
-        <v>62.221057891845703</v>
+        <v>61.821510314941399</v>
       </c>
       <c r="G11">
-        <v>46.0057838338154</v>
+        <v>45.539111481388197</v>
       </c>
       <c r="H11">
-        <v>56.906324157563297</v>
+        <v>56.6090505542683</v>
       </c>
       <c r="I11">
-        <v>66.061014277773396</v>
+        <v>65.825492417690199</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -2455,28 +2429,28 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>0.27618999999999999</v>
+        <v>0.27152999999999999</v>
       </c>
       <c r="C12">
-        <v>0.249949119357262</v>
+        <v>0.243903414081068</v>
       </c>
       <c r="D12">
-        <v>0.26965214436241902</v>
+        <v>0.26575450494874298</v>
       </c>
       <c r="E12">
-        <v>0.290849029152073</v>
+        <v>0.28534195008410501</v>
       </c>
       <c r="F12">
-        <v>62.614639282226598</v>
+        <v>62.248306274414098</v>
       </c>
       <c r="G12">
-        <v>56.383523171187903</v>
+        <v>56.113949107400899</v>
       </c>
       <c r="H12">
-        <v>60.021430658660201</v>
+        <v>59.7421032988197</v>
       </c>
       <c r="I12">
-        <v>64.5266312100524</v>
+        <v>64.765208406416704</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -2484,28 +2458,28 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>1.7996000000000002E-2</v>
+        <v>1.7739000000000001E-2</v>
       </c>
       <c r="C13">
         <v>0</v>
       </c>
       <c r="D13">
-        <v>1.6458294814498401E-2</v>
+        <v>1.6286779197987301E-2</v>
       </c>
       <c r="E13">
-        <v>2.7778728592042001E-2</v>
+        <v>2.8126192759763802E-2</v>
       </c>
       <c r="F13">
-        <v>24.444412231445298</v>
+        <v>24.368366241455099</v>
       </c>
       <c r="G13">
         <v>0</v>
       </c>
       <c r="H13">
-        <v>22.753024208163101</v>
+        <v>22.8880007444425</v>
       </c>
       <c r="I13">
-        <v>36.645716165735998</v>
+        <v>38.150305932683501</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -2513,28 +2487,28 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>1.0208999999999999E-2</v>
+        <v>1.0019E-2</v>
       </c>
       <c r="C14">
         <v>0</v>
       </c>
       <c r="D14">
-        <v>1.2913271909399299E-2</v>
+        <v>1.2224404004360199E-2</v>
       </c>
       <c r="E14">
-        <v>2.9749398206575101E-2</v>
+        <v>2.8688213464804001E-2</v>
       </c>
       <c r="F14">
-        <v>11.4526567459106</v>
+        <v>11.4016227722168</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
       <c r="H14">
-        <v>12.292681734733099</v>
+        <v>11.9101577121092</v>
       </c>
       <c r="I14">
-        <v>28.707866158606901</v>
+        <v>29.023567870432</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -2551,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>1.49570114484212E-2</v>
+        <v>9.7053893119051302E-3</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -2563,7 +2537,7 @@
         <v>0</v>
       </c>
       <c r="I15">
-        <v>10.9784274185754</v>
+        <v>7.3412948615512601</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -2571,28 +2545,28 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>2.5714999999999998E-2</v>
+        <v>2.5259E-2</v>
       </c>
       <c r="C16">
-        <v>1.99950276646782E-2</v>
+        <v>1.8963047123910601E-2</v>
       </c>
       <c r="D16">
-        <v>2.7201115178474199E-2</v>
+        <v>2.63440129467599E-2</v>
       </c>
       <c r="E16">
-        <v>3.3347679660273702E-2</v>
+        <v>3.2501831569723E-2</v>
       </c>
       <c r="F16">
-        <v>21.885288238525401</v>
+        <v>21.765935897827099</v>
       </c>
       <c r="G16">
-        <v>17.234366577603399</v>
+        <v>16.328704277373401</v>
       </c>
       <c r="H16">
-        <v>23.259661432801401</v>
+        <v>23.085980980824999</v>
       </c>
       <c r="I16">
-        <v>28.317664290524</v>
+        <v>28.689680541750501</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
@@ -2600,28 +2574,28 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>0.13372000000000001</v>
+        <v>0.13147</v>
       </c>
       <c r="C17">
-        <v>0.121445616816951</v>
+        <v>0.118526492977024</v>
       </c>
       <c r="D17">
-        <v>0.131690179558557</v>
+        <v>0.12834615727761101</v>
       </c>
       <c r="E17">
-        <v>0.143961983559726</v>
+        <v>0.14029537059002101</v>
       </c>
       <c r="F17">
-        <v>48.403434753417997</v>
+        <v>48.131546020507798</v>
       </c>
       <c r="G17">
-        <v>43.7859269174375</v>
+        <v>43.752198136054602</v>
       </c>
       <c r="H17">
-        <v>47.659151055029199</v>
+        <v>47.336859663417599</v>
       </c>
       <c r="I17">
-        <v>51.2023384483455</v>
+        <v>51.272093459612002</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
@@ -2629,28 +2603,28 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>7.9016000000000003E-2</v>
+        <v>7.7701999999999993E-2</v>
       </c>
       <c r="C18">
-        <v>6.2506243759861704E-2</v>
+        <v>6.0351151506706897E-2</v>
       </c>
       <c r="D18">
-        <v>8.2579909230291099E-2</v>
+        <v>7.9819631369634894E-2</v>
       </c>
       <c r="E18">
-        <v>0.11248245186448</v>
+        <v>0.105898079185134</v>
       </c>
       <c r="F18">
-        <v>33.762077331542997</v>
+        <v>33.614978790283203</v>
       </c>
       <c r="G18">
-        <v>27.8722517392142</v>
+        <v>27.453008284809201</v>
       </c>
       <c r="H18">
-        <v>34.483906215391897</v>
+        <v>34.259798142338802</v>
       </c>
       <c r="I18">
-        <v>43.488958074206003</v>
+        <v>42.223504550012898</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
@@ -2658,28 +2632,28 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>0.26668999999999998</v>
+        <v>0.26212999999999997</v>
       </c>
       <c r="C19">
-        <v>0.23854606959522001</v>
+        <v>0.23149117816717099</v>
       </c>
       <c r="D19">
-        <v>0.26457099745941098</v>
+        <v>0.25718906621061499</v>
       </c>
       <c r="E19">
-        <v>0.29432382634886001</v>
+        <v>0.285797701017735</v>
       </c>
       <c r="F19">
-        <v>42.684177398681598</v>
+        <v>42.443317413330099</v>
       </c>
       <c r="G19">
-        <v>38.557335684736302</v>
+        <v>38.383814592002203</v>
       </c>
       <c r="H19">
-        <v>42.265043664806001</v>
+        <v>42.021859907041403</v>
       </c>
       <c r="I19">
-        <v>46.220780898084598</v>
+        <v>46.049561676141202</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
@@ -2687,28 +2661,28 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>0.32463999999999998</v>
+        <v>0.31869999999999998</v>
       </c>
       <c r="C20">
-        <v>0.26339716916921702</v>
+        <v>0.26972291058796</v>
       </c>
       <c r="D20">
-        <v>0.32427269851795498</v>
+        <v>0.317156361390946</v>
       </c>
       <c r="E20">
-        <v>0.38018580232136201</v>
+        <v>0.37677641061960199</v>
       </c>
       <c r="F20">
-        <v>37.400825500488303</v>
+        <v>37.157894134521499</v>
       </c>
       <c r="G20">
-        <v>31.124524537394301</v>
+        <v>32.089928989067701</v>
       </c>
       <c r="H20">
-        <v>37.256413844566197</v>
+        <v>37.1108245774994</v>
       </c>
       <c r="I20">
-        <v>41.993149852602102</v>
+        <v>42.047787661262099</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
@@ -2716,28 +2690,28 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>0.92530000000000001</v>
+        <v>0.90944999999999998</v>
       </c>
       <c r="C21">
-        <v>0.75779603642637805</v>
+        <v>0.74990808558618505</v>
       </c>
       <c r="D21">
-        <v>0.908776334276164</v>
+        <v>0.89324382284036197</v>
       </c>
       <c r="E21">
-        <v>1.00650103235766</v>
+        <v>0.98987306672381503</v>
       </c>
       <c r="F21">
-        <v>40.746803283691399</v>
+        <v>40.515853881835902</v>
       </c>
       <c r="G21">
-        <v>35.135661161398701</v>
+        <v>35.086673203065402</v>
       </c>
       <c r="H21">
-        <v>40.592128492153599</v>
+        <v>40.525104066959003</v>
       </c>
       <c r="I21">
-        <v>44.464224851103197</v>
+        <v>44.2049677962817</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
@@ -2754,7 +2728,7 @@
         <v>0</v>
       </c>
       <c r="E22">
-        <v>1.1609821487602E-2</v>
+        <v>1.3516433608454E-2</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -2766,7 +2740,7 @@
         <v>0</v>
       </c>
       <c r="I22">
-        <v>8.5623481922499103</v>
+        <v>11.2234070318801</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
@@ -2774,28 +2748,28 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>0.10441</v>
+        <v>0.10219</v>
       </c>
       <c r="C23">
-        <v>5.2548451818347899E-2</v>
+        <v>4.9736920665734999E-2</v>
       </c>
       <c r="D23">
-        <v>0.117534720018192</v>
+        <v>0.11106860875815699</v>
       </c>
       <c r="E23">
-        <v>0.183292603061085</v>
+        <v>0.173401009044301</v>
       </c>
       <c r="F23">
-        <v>15.8743944168091</v>
+        <v>15.762010574340801</v>
       </c>
       <c r="G23">
-        <v>7.9661265640605698</v>
+        <v>8.0388688949169502</v>
       </c>
       <c r="H23">
-        <v>17.760657273084</v>
+        <v>17.505233479874502</v>
       </c>
       <c r="I23">
-        <v>27.160334333359199</v>
+        <v>26.848275316707699</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
@@ -2803,28 +2777,28 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>8.7363000000000007E-3</v>
+        <v>8.5991000000000001E-3</v>
       </c>
       <c r="C24">
-        <v>5.0212822500287496E-3</v>
+        <v>5.0037841873113399E-3</v>
       </c>
       <c r="D24">
-        <v>8.3425677472911703E-3</v>
+        <v>8.3678669516756808E-3</v>
       </c>
       <c r="E24">
-        <v>1.40650964801562E-2</v>
+        <v>1.33651515221934E-2</v>
       </c>
       <c r="F24">
-        <v>52.778224945068402</v>
+        <v>52.596385955810497</v>
       </c>
       <c r="G24">
-        <v>36.834043276985902</v>
+        <v>36.405512001672101</v>
       </c>
       <c r="H24">
-        <v>52.722471548077898</v>
+        <v>54.108612674577799</v>
       </c>
       <c r="I24">
-        <v>73.136289003193596</v>
+        <v>71.590742356574395</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
@@ -2841,7 +2815,7 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>1.7586872306850399E-2</v>
+        <v>8.3927117982084392E-3</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -2853,7 +2827,7 @@
         <v>0</v>
       </c>
       <c r="I25">
-        <v>6.11259354167011</v>
+        <v>3.1670935027742999</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
@@ -2861,28 +2835,28 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>2.6272000000000001E-3</v>
+        <v>2.5912999999999999E-3</v>
       </c>
       <c r="C26">
         <v>0</v>
       </c>
       <c r="D26">
-        <v>2.1496363305911199E-3</v>
+        <v>2.1981228534132002E-3</v>
       </c>
       <c r="E26">
-        <v>6.0920522397118603E-3</v>
+        <v>5.3548985708279503E-3</v>
       </c>
       <c r="F26">
-        <v>12.838894844055201</v>
+        <v>12.7884817123413</v>
       </c>
       <c r="G26">
         <v>0</v>
       </c>
       <c r="H26">
-        <v>12.547413575952699</v>
+        <v>13.095995884035</v>
       </c>
       <c r="I26">
-        <v>33.786747665410601</v>
+        <v>32.824932401081199</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
@@ -2890,28 +2864,28 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>1.1691999999999999E-2</v>
+        <v>1.1424999999999999E-2</v>
       </c>
       <c r="C27">
-        <v>7.4400805483478896E-3</v>
+        <v>8.0575417494308191E-3</v>
       </c>
       <c r="D27">
-        <v>1.0446590222781001E-2</v>
+        <v>1.02734447143371E-2</v>
       </c>
       <c r="E27">
-        <v>2.54675012677835E-2</v>
+        <v>1.9088535890067201E-2</v>
       </c>
       <c r="F27">
-        <v>8.9512510299682599</v>
+        <v>8.8443851470947301</v>
       </c>
       <c r="G27">
-        <v>5.9240175536727602</v>
+        <v>6.1667220164440302</v>
       </c>
       <c r="H27">
-        <v>8.7142828459259594</v>
+        <v>8.4784117414991798</v>
       </c>
       <c r="I27">
-        <v>16.428072438263101</v>
+        <v>14.2798210020767</v>
       </c>
     </row>
   </sheetData>
@@ -2920,7 +2894,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9AB23250-6E26-4123-A1E0-E87711280CB9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4C52509-FF49-496E-B77E-F690C78D3575}">
   <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -2958,28 +2932,28 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.15697</v>
+        <v>0.23488999999999999</v>
       </c>
       <c r="C2">
-        <v>0.107312381726358</v>
+        <v>0.19963043234064201</v>
       </c>
       <c r="D2">
-        <v>0.15875246080457101</v>
+        <v>0.22685944570550801</v>
       </c>
       <c r="E2">
-        <v>0.21802065841910201</v>
+        <v>0.25147759333615399</v>
       </c>
       <c r="F2">
-        <v>15.3373670578003</v>
+        <v>22.3976726531982</v>
       </c>
       <c r="G2">
-        <v>10.596543514204701</v>
+        <v>19.063461420646998</v>
       </c>
       <c r="H2">
-        <v>15.066087385122399</v>
+        <v>22.0841525804586</v>
       </c>
       <c r="I2">
-        <v>20.910432791461801</v>
+        <v>24.859297646855399</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -2987,28 +2961,28 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1.3868E-2</v>
+        <v>6.2796000000000005E-2</v>
       </c>
       <c r="C3">
-        <v>6.6078156384741004E-3</v>
+        <v>4.2670052925466703E-2</v>
       </c>
       <c r="D3">
-        <v>1.68250522197896E-2</v>
+        <v>6.7135447235371307E-2</v>
       </c>
       <c r="E3">
-        <v>3.0961818210359499E-2</v>
+        <v>9.0260107082445903E-2</v>
       </c>
       <c r="F3">
-        <v>4.11454057693481</v>
+        <v>16.526607513427699</v>
       </c>
       <c r="G3">
-        <v>1.5328164341942401</v>
+        <v>11.016109038447899</v>
       </c>
       <c r="H3">
-        <v>4.49983404916245</v>
+        <v>17.4465461228957</v>
       </c>
       <c r="I3">
-        <v>7.8656725126124103</v>
+        <v>23.701346653169001</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -3016,28 +2990,28 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1.9774E-2</v>
+        <v>4.0495999999999997E-2</v>
       </c>
       <c r="C4">
-        <v>1.46565446392131E-2</v>
+        <v>3.2087517446786701E-2</v>
       </c>
       <c r="D4">
-        <v>2.06057073783854E-2</v>
+        <v>3.7988686881925103E-2</v>
       </c>
       <c r="E4">
-        <v>2.5886891655145901E-2</v>
+        <v>4.2956621831309501E-2</v>
       </c>
       <c r="F4">
-        <v>12.988462448120099</v>
+        <v>25.6166667938232</v>
       </c>
       <c r="G4">
-        <v>8.9349334946849606</v>
+        <v>20.341318704245801</v>
       </c>
       <c r="H4">
-        <v>13.0327455628285</v>
+        <v>24.5339233423236</v>
       </c>
       <c r="I4">
-        <v>16.945326762255899</v>
+        <v>28.2568439311978</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -3045,28 +3019,28 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>3.6138999999999998E-2</v>
+        <v>7.1240999999999999E-2</v>
       </c>
       <c r="C5">
-        <v>2.3852039125490301E-2</v>
+        <v>5.6000443024226201E-2</v>
       </c>
       <c r="D5">
-        <v>3.6012545271361503E-2</v>
+        <v>6.5031732499950007E-2</v>
       </c>
       <c r="E5">
-        <v>5.15098378769967E-2</v>
+        <v>7.2573974659545806E-2</v>
       </c>
       <c r="F5">
-        <v>16.112239837646499</v>
+        <v>31.015975952148398</v>
       </c>
       <c r="G5">
-        <v>10.408615705012201</v>
+        <v>25.349250761903701</v>
       </c>
       <c r="H5">
-        <v>15.895562837995501</v>
+        <v>29.440663667016299</v>
       </c>
       <c r="I5">
-        <v>22.8200911228409</v>
+        <v>32.323953527038697</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -3074,28 +3048,28 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>0.14865</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>9.0864865217903601E-2</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>0.14790998016582499</v>
       </c>
       <c r="E6">
-        <v>3.78041632437289E-2</v>
+        <v>0.185798819467969</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>24.750299453735401</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>14.451154254545401</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>25.186996193493801</v>
       </c>
       <c r="I6">
-        <v>5.7725052956234304</v>
+        <v>33.210504930091801</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -3103,28 +3077,28 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>7.8481000000000002E-3</v>
+        <v>2.0521999999999999E-2</v>
       </c>
       <c r="C7">
-        <v>1.2252118822644201E-3</v>
+        <v>1.2565138680808999E-2</v>
       </c>
       <c r="D7">
-        <v>7.6126124376393496E-3</v>
+        <v>1.7924211418907401E-2</v>
       </c>
       <c r="E7">
-        <v>1.38932607948916E-2</v>
+        <v>2.3665034894464899E-2</v>
       </c>
       <c r="F7">
-        <v>19.315050125122099</v>
+        <v>51.015132904052699</v>
       </c>
       <c r="G7">
-        <v>3.9014542767545501</v>
+        <v>31.346833945540698</v>
       </c>
       <c r="H7">
-        <v>18.946128606703802</v>
+        <v>47.722648557947402</v>
       </c>
       <c r="I7">
-        <v>33.001348761834002</v>
+        <v>64.627576146343898</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
@@ -3132,28 +3106,28 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>2.4778999999999999E-2</v>
+        <v>3.6142000000000001E-2</v>
       </c>
       <c r="C8">
-        <v>1.6087942221397301E-2</v>
+        <v>2.43043362489723E-2</v>
       </c>
       <c r="D8">
-        <v>2.3783260260949901E-2</v>
+        <v>3.25135123555957E-2</v>
       </c>
       <c r="E8">
-        <v>3.06916614145623E-2</v>
+        <v>4.1597943835704899E-2</v>
       </c>
       <c r="F8">
-        <v>25.753686904907202</v>
+        <v>37.555858612060497</v>
       </c>
       <c r="G8">
-        <v>17.195154713498798</v>
+        <v>26.5341071849932</v>
       </c>
       <c r="H8">
-        <v>24.731481049714301</v>
+        <v>34.788934170252197</v>
       </c>
       <c r="I8">
-        <v>32.765004652705599</v>
+        <v>43.464916584245699</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
@@ -3161,28 +3135,28 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>1.3206000000000001E-2</v>
+        <v>1.4389000000000001E-2</v>
       </c>
       <c r="C9">
-        <v>9.4123470667229394E-3</v>
+        <v>1.0036956729387699E-2</v>
       </c>
       <c r="D9">
-        <v>1.2690300602764101E-2</v>
+        <v>1.30075017205386E-2</v>
       </c>
       <c r="E9">
-        <v>1.5212763727603801E-2</v>
+        <v>1.6530919842645101E-2</v>
       </c>
       <c r="F9">
-        <v>29.301378250122099</v>
+        <v>31.903781890869102</v>
       </c>
       <c r="G9">
-        <v>21.638547426826499</v>
+        <v>22.637318574811101</v>
       </c>
       <c r="H9">
-        <v>27.963364751617402</v>
+        <v>29.701379352175</v>
       </c>
       <c r="I9">
-        <v>34.638153801647299</v>
+        <v>37.491551213080101</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -3190,28 +3164,28 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>4.4248999999999997E-2</v>
+        <v>4.2523999999999999E-2</v>
       </c>
       <c r="C10">
-        <v>3.1392496275139702E-2</v>
+        <v>2.6363265455237601E-2</v>
       </c>
       <c r="D10">
-        <v>4.3056851989326399E-2</v>
+        <v>3.73587247034552E-2</v>
       </c>
       <c r="E10">
-        <v>5.4119979678719697E-2</v>
+        <v>4.8882018469087803E-2</v>
       </c>
       <c r="F10">
-        <v>35.760456085205099</v>
+        <v>34.608566284179702</v>
       </c>
       <c r="G10">
-        <v>25.6576566989167</v>
+        <v>21.578549282794501</v>
       </c>
       <c r="H10">
-        <v>34.8261922366449</v>
+        <v>31.126729431069599</v>
       </c>
       <c r="I10">
-        <v>43.832958740844703</v>
+        <v>41.338855178330299</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -3219,28 +3193,28 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>7.3383000000000004E-2</v>
+        <v>8.3709000000000006E-3</v>
       </c>
       <c r="C11">
-        <v>6.0423190496512798E-2</v>
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>7.6078711794962797E-2</v>
+        <v>1.1762622537734401E-2</v>
       </c>
       <c r="E11">
-        <v>9.2535040802279103E-2</v>
+        <v>4.6498260342207699E-2</v>
       </c>
       <c r="F11">
-        <v>25.346965789794901</v>
+        <v>3.3123333454132098</v>
       </c>
       <c r="G11">
-        <v>20.3014523788713</v>
+        <v>0</v>
       </c>
       <c r="H11">
-        <v>25.447385981222801</v>
+        <v>3.9901858543359698</v>
       </c>
       <c r="I11">
-        <v>29.8345582137203</v>
+        <v>17.285938862056199</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -3248,28 +3222,28 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>9.4244999999999995E-2</v>
+        <v>0</v>
       </c>
       <c r="C12">
-        <v>8.0598850246135001E-2</v>
+        <v>0</v>
       </c>
       <c r="D12">
-        <v>9.7366837520197896E-2</v>
+        <v>5.2494434690360204E-4</v>
       </c>
       <c r="E12">
-        <v>0.10872408894270499</v>
+        <v>3.4003899668505998E-2</v>
       </c>
       <c r="F12">
-        <v>22.1390190124512</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>17.769887533296799</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>21.529260107760098</v>
+        <v>0.11509129392426699</v>
       </c>
       <c r="I12">
-        <v>24.505251038277901</v>
+        <v>7.5827838156299201</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -3277,28 +3251,28 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>1.1165000000000001E-3</v>
+        <v>3.7886999999999997E-2</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>2.26799133348486E-2</v>
       </c>
       <c r="D13">
-        <v>1.3355078088327899E-3</v>
+        <v>3.4628745673105199E-2</v>
       </c>
       <c r="E13">
-        <v>3.83966111474272E-2</v>
+        <v>4.70602680414497E-2</v>
       </c>
       <c r="F13">
-        <v>1.30733382701874</v>
+        <v>48.792568206787102</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>33.135708474559301</v>
       </c>
       <c r="H13">
-        <v>1.8068371072340501</v>
+        <v>46.799320695305397</v>
       </c>
       <c r="I13">
-        <v>40.602268210963501</v>
+        <v>59.981997836413903</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -3306,28 +3280,28 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>2.7564999999999999E-2</v>
+        <v>5.6349999999999997E-2</v>
       </c>
       <c r="C14">
-        <v>1.44876236680852E-2</v>
+        <v>2.5689879872719399E-2</v>
       </c>
       <c r="D14">
-        <v>2.6770563982347399E-2</v>
+        <v>4.7106585966760699E-2</v>
       </c>
       <c r="E14">
-        <v>5.99004555658567E-2</v>
+        <v>6.8947441862597797E-2</v>
       </c>
       <c r="F14">
-        <v>23.842178344726602</v>
+        <v>51.681430816650398</v>
       </c>
       <c r="G14">
-        <v>14.439348915305301</v>
+        <v>28.488263445929899</v>
       </c>
       <c r="H14">
-        <v>25.3886412449639</v>
+        <v>45.9614075874387</v>
       </c>
       <c r="I14">
-        <v>51.521388540920697</v>
+        <v>58.539026981120799</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -3335,28 +3309,28 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>8.0045000000000005E-2</v>
+        <v>4.4950999999999998E-2</v>
       </c>
       <c r="C15">
-        <v>5.9736000471431898E-2</v>
+        <v>1.7294485711214599E-2</v>
       </c>
       <c r="D15">
-        <v>7.8952403416861494E-2</v>
+        <v>3.8449698196749899E-2</v>
       </c>
       <c r="E15">
-        <v>9.7744580127846703E-2</v>
+        <v>5.42932040564773E-2</v>
       </c>
       <c r="F15">
-        <v>58.216335296630902</v>
+        <v>33.2401733398438</v>
       </c>
       <c r="G15">
-        <v>47.421112708621003</v>
+        <v>13.429057859561301</v>
       </c>
       <c r="H15">
-        <v>60.5598341664505</v>
+        <v>29.720137743848898</v>
       </c>
       <c r="I15">
-        <v>70.762217700571497</v>
+        <v>44.103883591424903</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -3364,28 +3338,28 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>5.3983999999999997E-2</v>
+        <v>2.2709E-2</v>
       </c>
       <c r="C16">
-        <v>4.6510968504932797E-2</v>
+        <v>1.3188785073225901E-2</v>
       </c>
       <c r="D16">
-        <v>5.2215331931409301E-2</v>
+        <v>2.1016245050599201E-2</v>
       </c>
       <c r="E16">
-        <v>6.1081463407054101E-2</v>
+        <v>2.7116320309022501E-2</v>
       </c>
       <c r="F16">
-        <v>44.713138580322301</v>
+        <v>19.266616821289102</v>
       </c>
       <c r="G16">
-        <v>40.875656218469203</v>
+        <v>11.677636246294099</v>
       </c>
       <c r="H16">
-        <v>44.561158893633902</v>
+        <v>18.254712104246</v>
       </c>
       <c r="I16">
-        <v>50.785789602498298</v>
+        <v>23.836204028746501</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
@@ -3393,28 +3367,28 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>8.9552000000000007E-2</v>
+        <v>1.5218000000000001E-2</v>
       </c>
       <c r="C17">
-        <v>7.9878292573061394E-2</v>
+        <v>1.0572405741068399E-2</v>
       </c>
       <c r="D17">
-        <v>8.9703457727673602E-2</v>
+        <v>1.8297947985806501E-2</v>
       </c>
       <c r="E17">
-        <v>9.69699053180193E-2</v>
+        <v>2.50784283189311E-2</v>
       </c>
       <c r="F17">
-        <v>32.897514343261697</v>
+        <v>6.0434145927429199</v>
       </c>
       <c r="G17">
-        <v>28.931368617190699</v>
+        <v>3.8778682316528101</v>
       </c>
       <c r="H17">
-        <v>32.415252873879602</v>
+        <v>6.7776057996326999</v>
       </c>
       <c r="I17">
-        <v>34.831533529948103</v>
+        <v>9.3215167504737995</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
@@ -3422,28 +3396,28 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>0.11650000000000001</v>
+        <v>4.1134999999999998E-2</v>
       </c>
       <c r="C18">
-        <v>9.1826076038242194E-2</v>
+        <v>2.1303766495015201E-2</v>
       </c>
       <c r="D18">
-        <v>0.112989753947561</v>
+        <v>3.72328442942437E-2</v>
       </c>
       <c r="E18">
-        <v>0.13300471501501401</v>
+        <v>5.6889263830811901E-2</v>
       </c>
       <c r="F18">
-        <v>48.512245178222699</v>
+        <v>17.722339630126999</v>
       </c>
       <c r="G18">
-        <v>39.818195503391401</v>
+        <v>8.6647052506583293</v>
       </c>
       <c r="H18">
-        <v>47.2454457039712</v>
+        <v>15.8166324817172</v>
       </c>
       <c r="I18">
-        <v>53.152676863468301</v>
+        <v>25.115528815108998</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
@@ -3451,28 +3425,28 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>0.22559000000000001</v>
+        <v>4.5600000000000002E-2</v>
       </c>
       <c r="C19">
-        <v>0.20198051916607701</v>
+        <v>3.09306189015096E-2</v>
       </c>
       <c r="D19">
-        <v>0.22469852781923499</v>
+        <v>4.9413006168001601E-2</v>
       </c>
       <c r="E19">
-        <v>0.245348207517432</v>
+        <v>6.3679086141995495E-2</v>
       </c>
       <c r="F19">
-        <v>36.4697265625</v>
+        <v>7.8198194503784197</v>
       </c>
       <c r="G19">
-        <v>32.417369340368197</v>
+        <v>4.9375914836883901</v>
       </c>
       <c r="H19">
-        <v>36.135682175138697</v>
+        <v>8.0014162576235996</v>
       </c>
       <c r="I19">
-        <v>38.615757556742103</v>
+        <v>10.7437530147782</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
@@ -3480,28 +3454,28 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>0.33322000000000002</v>
+        <v>0</v>
       </c>
       <c r="C20">
-        <v>0.301310444047027</v>
+        <v>0</v>
       </c>
       <c r="D20">
-        <v>0.33277353589293401</v>
+        <v>0</v>
       </c>
       <c r="E20">
-        <v>0.373245920904693</v>
+        <v>3.2961717816749898E-2</v>
       </c>
       <c r="F20">
-        <v>39.000862121582003</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>33.648611790366303</v>
+        <v>0</v>
       </c>
       <c r="H20">
-        <v>38.293954236778099</v>
+        <v>0</v>
       </c>
       <c r="I20">
-        <v>42.659865924424501</v>
+        <v>3.7541484016303599</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
@@ -3509,28 +3483,28 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>0.70757000000000003</v>
+        <v>3.9618E-2</v>
       </c>
       <c r="C21">
-        <v>0.62084008403748303</v>
+        <v>2.27507101440141E-2</v>
       </c>
       <c r="D21">
-        <v>0.70928293406298504</v>
+        <v>7.8007895267882599E-2</v>
       </c>
       <c r="E21">
-        <v>0.79943621229370199</v>
+        <v>0.182775590068711</v>
       </c>
       <c r="F21">
-        <v>31.863374710083001</v>
+        <v>2.31804227828979</v>
       </c>
       <c r="G21">
-        <v>27.603953809492399</v>
+        <v>1.0472361699471899</v>
       </c>
       <c r="H21">
-        <v>31.664637931931502</v>
+        <v>3.5358146741990302</v>
       </c>
       <c r="I21">
-        <v>35.549033947583801</v>
+        <v>8.2779000769212701</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
@@ -3538,28 +3512,28 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>3.2800999999999997E-2</v>
+        <v>0</v>
       </c>
       <c r="C22">
-        <v>1.0563145873381899E-2</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>3.0761865541690199E-2</v>
+        <v>6.0172885742906598E-5</v>
       </c>
       <c r="E22">
-        <v>4.8737472655006303E-2</v>
+        <v>4.8996440539927598E-2</v>
       </c>
       <c r="F22">
-        <v>22.283037185668899</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>9.5703587717696408</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>23.0385507795596</v>
+        <v>4.6964191117408301E-2</v>
       </c>
       <c r="I22">
-        <v>35.968797453221498</v>
+        <v>43.337173262904301</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
@@ -3567,28 +3541,28 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>0.39953</v>
+        <v>0.11932</v>
       </c>
       <c r="C23">
-        <v>0.32557028164010698</v>
+        <v>4.3277544418866901E-2</v>
       </c>
       <c r="D23">
-        <v>0.38880239267062999</v>
+        <v>9.8922296557538203E-2</v>
       </c>
       <c r="E23">
-        <v>0.45585945168500902</v>
+        <v>0.162831648222025</v>
       </c>
       <c r="F23">
-        <v>59.518123626708999</v>
+        <v>18.148485183715799</v>
       </c>
       <c r="G23">
-        <v>53.4095469507212</v>
+        <v>6.5659706521085397</v>
       </c>
       <c r="H23">
-        <v>58.787127661302499</v>
+        <v>15.2043473516039</v>
       </c>
       <c r="I23">
-        <v>65.1726511152943</v>
+        <v>25.814954592834798</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
@@ -3596,28 +3570,28 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>1.0692E-3</v>
+        <v>0</v>
       </c>
       <c r="C24">
-        <v>9.7209047822205896E-5</v>
+        <v>0</v>
       </c>
       <c r="D24">
-        <v>1.5178765866393901E-3</v>
+        <v>0</v>
       </c>
       <c r="E24">
-        <v>2.5867137005680498E-3</v>
+        <v>1.6970154301329001E-3</v>
       </c>
       <c r="F24">
-        <v>7.9108862876892099</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>0.638388636323031</v>
+        <v>0</v>
       </c>
       <c r="H24">
-        <v>9.4764257393180795</v>
+        <v>0</v>
       </c>
       <c r="I24">
-        <v>15.2564267533785</v>
+        <v>12.0765886180907</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
@@ -3625,28 +3599,28 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>0.11854000000000001</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>7.0078608890175101E-2</v>
       </c>
       <c r="D25">
-        <v>1.7342255701432299E-4</v>
+        <v>0.103052792089583</v>
       </c>
       <c r="E25">
-        <v>2.9579690218314602E-3</v>
+        <v>0.137959204738721</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>42.484241485595703</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>26.202461159849999</v>
       </c>
       <c r="H25">
-        <v>6.7355143958303595E-2</v>
+        <v>39.183501208387902</v>
       </c>
       <c r="I25">
-        <v>1.14337231319446</v>
+        <v>52.445452943874798</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
@@ -3660,22 +3634,22 @@
         <v>0</v>
       </c>
       <c r="D26">
-        <v>0</v>
+        <v>1.14190611484392E-3</v>
       </c>
       <c r="E26">
-        <v>7.1991587196052202E-4</v>
+        <v>3.98721709941604E-3</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>3.4859459400177002</v>
       </c>
       <c r="G26">
         <v>0</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>6.6947303648474303</v>
       </c>
       <c r="I26">
-        <v>5.0403520480119299</v>
+        <v>31.165053353308799</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
@@ -3683,28 +3657,28 @@
         <v>26</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>5.5069000000000003E-3</v>
       </c>
       <c r="C27">
         <v>0</v>
       </c>
       <c r="D27">
-        <v>2.8678369212052499E-4</v>
+        <v>5.3076818237718501E-3</v>
       </c>
       <c r="E27">
-        <v>5.1041020247581202E-3</v>
+        <v>2.2292146123549999E-2</v>
       </c>
       <c r="F27">
-        <v>9.8524682223796803E-2</v>
+        <v>5.5233931541442898</v>
       </c>
       <c r="G27">
         <v>0</v>
       </c>
       <c r="H27">
-        <v>0.22537541411537401</v>
+        <v>4.4754929894455104</v>
       </c>
       <c r="I27">
-        <v>3.7598584880539301</v>
+        <v>17.842732986219801</v>
       </c>
     </row>
   </sheetData>
@@ -3713,7 +3687,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1661603-382E-4C71-B96B-FBA7988FD03B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80BC2D82-D24D-469A-8500-0436A91CF7D6}">
   <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -3751,28 +3725,28 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>4.7763E-2</v>
+        <v>0.15464</v>
       </c>
       <c r="C2">
-        <v>4.14958804418986E-2</v>
+        <v>0.111953644800367</v>
       </c>
       <c r="D2">
-        <v>6.2064701808343302E-2</v>
+        <v>0.157536590401717</v>
       </c>
       <c r="E2">
-        <v>9.0725782115768303E-2</v>
+        <v>0.216919635901896</v>
       </c>
       <c r="F2">
-        <v>4.8652148246765101</v>
+        <v>15.388108253479</v>
       </c>
       <c r="G2">
-        <v>3.7850361917865301</v>
+        <v>11.0711580014995</v>
       </c>
       <c r="H2">
-        <v>5.9218834424164504</v>
+        <v>15.2222147192108</v>
       </c>
       <c r="I2">
-        <v>9.1886870870717008</v>
+        <v>21.318299985949501</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -3780,28 +3754,28 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>4.9519000000000001E-2</v>
+        <v>1.3712E-2</v>
       </c>
       <c r="C3">
-        <v>2.4521330130846401E-2</v>
+        <v>2.82582963934101E-3</v>
       </c>
       <c r="D3">
-        <v>4.5726754889669999E-2</v>
+        <v>1.6850889182910299E-2</v>
       </c>
       <c r="E3">
-        <v>6.3152136430339803E-2</v>
+        <v>2.9841718511608301E-2</v>
       </c>
       <c r="F3">
-        <v>13.2411890029907</v>
+        <v>4.1315212249755904</v>
       </c>
       <c r="G3">
-        <v>5.8535433996342503</v>
+        <v>0.73483980883247502</v>
       </c>
       <c r="H3">
-        <v>11.9727974150272</v>
+        <v>4.5469512841053996</v>
       </c>
       <c r="I3">
-        <v>16.466061265345999</v>
+        <v>7.7425691413745801</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -3809,28 +3783,28 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>4.1062E-3</v>
+        <v>1.949E-2</v>
       </c>
       <c r="C4">
-        <v>3.6753263420628199E-3</v>
+        <v>1.53276865082789E-2</v>
       </c>
       <c r="D4">
-        <v>7.4537798801904897E-3</v>
+        <v>2.0654208367646799E-2</v>
       </c>
       <c r="E4">
-        <v>1.1762598510690701E-2</v>
+        <v>2.6797819451669799E-2</v>
       </c>
       <c r="F4">
-        <v>2.9201712608337398</v>
+        <v>13.0364217758179</v>
       </c>
       <c r="G4">
-        <v>2.2820734402115299</v>
+        <v>9.6873290687479905</v>
       </c>
       <c r="H4">
-        <v>4.6833738204219797</v>
+        <v>13.282681944520199</v>
       </c>
       <c r="I4">
-        <v>7.5141299101336099</v>
+        <v>17.476506090821601</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -3838,28 +3812,28 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>7.2915000000000002E-3</v>
+        <v>3.5603000000000003E-2</v>
       </c>
       <c r="C5">
-        <v>6.0383422778822297E-3</v>
+        <v>2.54135597432728E-2</v>
       </c>
       <c r="D5">
-        <v>1.03262447313631E-2</v>
+        <v>3.58201951807844E-2</v>
       </c>
       <c r="E5">
-        <v>1.86806029570343E-2</v>
+        <v>5.4669047779170699E-2</v>
       </c>
       <c r="F5">
-        <v>3.4945025444030802</v>
+        <v>16.171260833740199</v>
       </c>
       <c r="G5">
-        <v>2.6112225651885801</v>
+        <v>11.5882719833303</v>
       </c>
       <c r="H5">
-        <v>4.4955633867977598</v>
+        <v>16.146275873463299</v>
       </c>
       <c r="I5">
-        <v>8.54838503070361</v>
+        <v>24.177513573868499</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
@@ -3867,28 +3841,28 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>7.2369000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="C6">
-        <v>4.2664469505925E-2</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>7.0984248565527902E-2</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>0.10326844175177</v>
+        <v>3.6725948142646098E-2</v>
       </c>
       <c r="F6">
-        <v>11.682695388793899</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>7.1774574479406903</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>11.721370767441201</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>16.835976724203601</v>
+        <v>5.6052040448319502</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -3896,28 +3870,28 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>4.8853999999999998E-3</v>
+        <v>7.7247000000000001E-3</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>1.0892563763506601E-3</v>
       </c>
       <c r="D7">
-        <v>2.4983779763057602E-3</v>
+        <v>7.48176042217136E-3</v>
       </c>
       <c r="E7">
-        <v>9.2862615767213292E-3</v>
+        <v>1.5220824474087701E-2</v>
       </c>
       <c r="F7">
-        <v>12.969240188598601</v>
+        <v>19.380681991577099</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>3.43740689852965</v>
       </c>
       <c r="H7">
-        <v>7.0620003330654004</v>
+        <v>19.082095093987402</v>
       </c>
       <c r="I7">
-        <v>25.506569092955001</v>
+        <v>34.9012405188044</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
@@ -3925,28 +3899,28 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>2.4409E-2</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>1.71899449163921E-2</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>2.3974549757339501E-2</v>
       </c>
       <c r="E8">
-        <v>2.86304844126013E-3</v>
+        <v>3.16034388215908E-2</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>25.857662200927699</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>17.614151863653301</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>25.4128627609633</v>
       </c>
       <c r="I8">
-        <v>3.2534500398035902</v>
+        <v>34.951826553011799</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
@@ -3954,28 +3928,28 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>1.3008E-2</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>9.6931847145354695E-3</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>1.2629725177092399E-2</v>
       </c>
       <c r="E9">
-        <v>1.2302316962531201E-3</v>
+        <v>1.5395375106494901E-2</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>29.410943984985401</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>21.863986539993601</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>28.3643614068727</v>
       </c>
       <c r="I9">
-        <v>3.0432673068057801</v>
+        <v>36.087416369307398</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
@@ -3983,28 +3957,28 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>4.3550999999999999E-2</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>3.0632823460484699E-2</v>
       </c>
       <c r="D10">
-        <v>1.3615194752635599E-3</v>
+        <v>4.28177888268104E-2</v>
       </c>
       <c r="E10">
-        <v>7.0064149980138199E-3</v>
+        <v>5.4178549438205797E-2</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>35.883804321289098</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>25.782460597135302</v>
       </c>
       <c r="H10">
-        <v>1.1080124454704301</v>
+        <v>35.145301269588799</v>
       </c>
       <c r="I10">
-        <v>5.8605757380928498</v>
+        <v>45.709143597331497</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
@@ -4012,28 +3986,28 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>7.2343000000000005E-2</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>5.9163207244021999E-2</v>
       </c>
       <c r="D11">
-        <v>1.2140260668095501E-2</v>
+        <v>7.4831954190651098E-2</v>
       </c>
       <c r="E11">
-        <v>3.46218794828645E-2</v>
+        <v>9.4171844236254701E-2</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>25.456565856933601</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>19.940602353640401</v>
       </c>
       <c r="H11">
-        <v>4.1961803609093904</v>
+        <v>25.607802431859401</v>
       </c>
       <c r="I11">
-        <v>11.228369184858099</v>
+        <v>30.377289903725099</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -4041,28 +4015,28 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>1.0553E-2</v>
+        <v>9.2814999999999995E-2</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>7.43392537449242E-2</v>
       </c>
       <c r="D12">
-        <v>2.6480748589404499E-2</v>
+        <v>9.5709885129989306E-2</v>
       </c>
       <c r="E12">
-        <v>4.3826605873618203E-2</v>
+        <v>0.106005867306801</v>
       </c>
       <c r="F12">
-        <v>3.4190542697906499</v>
+        <v>22.198593139648398</v>
       </c>
       <c r="G12">
-        <v>0</v>
+        <v>17.188134106331098</v>
       </c>
       <c r="H12">
-        <v>5.8451657851700496</v>
+        <v>21.453350404956499</v>
       </c>
       <c r="I12">
-        <v>9.6949133287051392</v>
+        <v>24.2780484090196</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -4070,28 +4044,28 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>8.1709999999999994E-3</v>
+        <v>1.1004999999999999E-3</v>
       </c>
       <c r="C13">
-        <v>9.5475992356614404E-4</v>
+        <v>0</v>
       </c>
       <c r="D13">
-        <v>6.5673811375083898E-3</v>
+        <v>1.3327998070230601E-3</v>
       </c>
       <c r="E13">
-        <v>1.67816085172789E-2</v>
+        <v>3.4263242476177402E-2</v>
       </c>
       <c r="F13">
-        <v>10.390475273132299</v>
+        <v>1.3125017881393399</v>
       </c>
       <c r="G13">
-        <v>1.2086175163039199</v>
+        <v>0</v>
       </c>
       <c r="H13">
-        <v>8.7098401886739207</v>
+        <v>1.8429961646666</v>
       </c>
       <c r="I13">
-        <v>22.286326462259801</v>
+        <v>37.682240714308101</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
@@ -4099,28 +4073,28 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>7.7211000000000001E-4</v>
+        <v>2.7154999999999999E-2</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>1.45418876351537E-2</v>
       </c>
       <c r="D14">
-        <v>1.30617123534033E-16</v>
+        <v>2.6222054140889E-2</v>
       </c>
       <c r="E14">
-        <v>1.67664856322601E-2</v>
+        <v>5.9708400891201899E-2</v>
       </c>
       <c r="F14">
-        <v>1.4536426067352299</v>
+        <v>23.9347114562988</v>
       </c>
       <c r="G14">
-        <v>0</v>
+        <v>14.5265490712071</v>
       </c>
       <c r="H14">
-        <v>1.3679145077734499E-13</v>
+        <v>25.393545794520499</v>
       </c>
       <c r="I14">
-        <v>15.8590828457806</v>
+        <v>52.656769493924998</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
@@ -4128,28 +4102,28 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>9.8528999999999995E-3</v>
+        <v>7.8783000000000006E-2</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>5.8535569206022098E-2</v>
       </c>
       <c r="D15">
-        <v>6.12186064540538E-3</v>
+        <v>7.8191522152283505E-2</v>
       </c>
       <c r="E15">
-        <v>2.6120908821414501E-2</v>
+        <v>9.6982260939679807E-2</v>
       </c>
       <c r="F15">
-        <v>8.1688718795776403</v>
+        <v>58.432968139648402</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>48.4712235475697</v>
       </c>
       <c r="H15">
-        <v>4.8173279277812098</v>
+        <v>61.676809303917601</v>
       </c>
       <c r="I15">
-        <v>18.800616189715502</v>
+        <v>72.264859169624302</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
@@ -4157,28 +4131,28 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>9.4687999999999994E-3</v>
+        <v>5.3130999999999998E-2</v>
       </c>
       <c r="C16">
-        <v>4.2331367025911799E-3</v>
+        <v>4.6088803679182701E-2</v>
       </c>
       <c r="D16">
-        <v>7.9790800225469794E-3</v>
+        <v>5.1819637853125801E-2</v>
       </c>
       <c r="E16">
-        <v>1.2252965227112E-2</v>
+        <v>6.07451392595003E-2</v>
       </c>
       <c r="F16">
-        <v>8.3127498626709002</v>
+        <v>44.855091094970703</v>
       </c>
       <c r="G16">
-        <v>3.5050058745282802</v>
+        <v>40.844396960610702</v>
       </c>
       <c r="H16">
-        <v>6.82537089885746</v>
+        <v>45.325804201181299</v>
       </c>
       <c r="I16">
-        <v>10.3664098283817</v>
+        <v>51.665964813792897</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
@@ -4186,28 +4160,28 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>1.1993999999999999E-2</v>
+        <v>8.8166999999999995E-2</v>
       </c>
       <c r="C17">
-        <v>7.4138055693129196E-3</v>
+        <v>7.9111538571075599E-2</v>
       </c>
       <c r="D17">
-        <v>1.7962864012736401E-2</v>
+        <v>8.8461538067880693E-2</v>
       </c>
       <c r="E17">
-        <v>2.4477538604593702E-2</v>
+        <v>9.5819077303944497E-2</v>
       </c>
       <c r="F17">
-        <v>4.9208025932312003</v>
+        <v>32.993434906005902</v>
       </c>
       <c r="G17">
-        <v>2.7798362370095702</v>
+        <v>29.473914769845798</v>
       </c>
       <c r="H17">
-        <v>6.3827265853068296</v>
+        <v>32.509677416209897</v>
       </c>
       <c r="I17">
-        <v>8.7325786857511201</v>
+        <v>34.9007995489142</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
@@ -4215,28 +4189,28 @@
         <v>17</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>0.11468</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>8.9519797854043404E-2</v>
       </c>
       <c r="D18">
-        <v>2.2192086020185798E-3</v>
+        <v>0.111724629050044</v>
       </c>
       <c r="E18">
-        <v>1.49876506882036E-2</v>
+        <v>0.132605809571854</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>48.662681579589801</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>40.301337564110298</v>
       </c>
       <c r="H18">
-        <v>0.90655844569497102</v>
+        <v>47.820215024471302</v>
       </c>
       <c r="I18">
-        <v>6.0786118583548197</v>
+        <v>54.0527075085581</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
@@ -4244,28 +4218,28 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>2.7334000000000001E-2</v>
+        <v>0.22209000000000001</v>
       </c>
       <c r="C19">
-        <v>1.85422613910948E-2</v>
+        <v>0.19841429351737</v>
       </c>
       <c r="D19">
-        <v>3.7690275749106099E-2</v>
+        <v>0.22063133053060399</v>
       </c>
       <c r="E19">
-        <v>5.6666858425109601E-2</v>
+        <v>0.240795184785977</v>
       </c>
       <c r="F19">
-        <v>4.9783406257629403</v>
+        <v>36.579437255859403</v>
       </c>
       <c r="G19">
-        <v>3.0120442687381099</v>
+        <v>33.022210449296999</v>
       </c>
       <c r="H19">
-        <v>5.9640756107000996</v>
+        <v>36.1831047568446</v>
       </c>
       <c r="I19">
-        <v>9.19037179387648</v>
+        <v>38.556976088751902</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
@@ -4273,28 +4247,28 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>3.1501000000000001E-2</v>
+        <v>0.32797999999999999</v>
       </c>
       <c r="C20">
-        <v>1.4607943672055399E-2</v>
+        <v>0.29407709172256102</v>
       </c>
       <c r="D20">
-        <v>4.9432408949008598E-2</v>
+        <v>0.32658353737300999</v>
       </c>
       <c r="E20">
-        <v>7.5384444603741801E-2</v>
+        <v>0.36106436584014201</v>
       </c>
       <c r="F20">
-        <v>4.9909243583679199</v>
+        <v>39.114818572997997</v>
       </c>
       <c r="G20">
-        <v>1.7345120621557399</v>
+        <v>33.149756194082002</v>
       </c>
       <c r="H20">
-        <v>5.6825671140751703</v>
+        <v>38.266664242472601</v>
       </c>
       <c r="I20">
-        <v>8.6699168838131602</v>
+        <v>42.024600076746303</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
@@ -4302,28 +4276,28 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>0.19728000000000001</v>
+        <v>0.69645999999999997</v>
       </c>
       <c r="C21">
-        <v>9.3093953839829102E-2</v>
+        <v>0.59403578919636602</v>
       </c>
       <c r="D21">
-        <v>0.200237015978809</v>
+        <v>0.69830144829685903</v>
       </c>
       <c r="E21">
-        <v>0.237881595962639</v>
+        <v>0.77026217652410001</v>
       </c>
       <c r="F21">
-        <v>9.6223344802856392</v>
+        <v>31.9483642578125</v>
       </c>
       <c r="G21">
-        <v>4.2654281265428597</v>
+        <v>27.2491562912025</v>
       </c>
       <c r="H21">
-        <v>8.9669936464128206</v>
+        <v>31.821848923987901</v>
       </c>
       <c r="I21">
-        <v>10.8144268922329</v>
+        <v>35.035301108746303</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
@@ -4331,28 +4305,28 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>6.4809000000000005E-2</v>
+        <v>3.2254999999999999E-2</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>1.12548673007735E-2</v>
       </c>
       <c r="D22">
-        <v>4.2656826120739101E-2</v>
+        <v>3.0870808324895801E-2</v>
       </c>
       <c r="E22">
-        <v>6.8891008026512199E-2</v>
+        <v>4.7063401743097297E-2</v>
       </c>
       <c r="F22">
-        <v>46.020206451416001</v>
+        <v>22.332128524780298</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>9.8026531682378</v>
       </c>
       <c r="H22">
-        <v>33.106624725051901</v>
+        <v>23.624913976043501</v>
       </c>
       <c r="I22">
-        <v>46.338951969071204</v>
+        <v>34.948592020889301</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
@@ -4360,28 +4334,28 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>9.7234999999999995E-3</v>
+        <v>0.39328999999999997</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>0.32354349537661398</v>
       </c>
       <c r="D23">
-        <v>1.15564212335261E-2</v>
+        <v>0.38208707731693597</v>
       </c>
       <c r="E23">
-        <v>5.5277779032587897E-2</v>
+        <v>0.45125540939848302</v>
       </c>
       <c r="F23">
-        <v>2.2761332988739</v>
+        <v>59.728923797607401</v>
       </c>
       <c r="G23">
-        <v>0</v>
+        <v>53.820665808183598</v>
       </c>
       <c r="H23">
-        <v>1.7796387844366199</v>
+        <v>59.257361569093199</v>
       </c>
       <c r="I23">
-        <v>8.2442059523547595</v>
+        <v>65.752440409967704</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
@@ -4389,28 +4363,28 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>2.8115000000000002E-3</v>
+        <v>1.0544E-3</v>
       </c>
       <c r="C24">
-        <v>7.7536013125919102E-4</v>
+        <v>1.3154089347766599E-6</v>
       </c>
       <c r="D24">
-        <v>2.7217119475285499E-3</v>
+        <v>1.4228123081172499E-3</v>
       </c>
       <c r="E24">
-        <v>4.5755417250720699E-3</v>
+        <v>2.4030986520861301E-3</v>
       </c>
       <c r="F24">
-        <v>20.076982498168899</v>
+        <v>7.9177985191345197</v>
       </c>
       <c r="G24">
-        <v>4.4143350606866401</v>
+        <v>9.1776177832069393E-3</v>
       </c>
       <c r="H24">
-        <v>17.5531965810667</v>
+        <v>8.9521166674988599</v>
       </c>
       <c r="I24">
-        <v>30.1522011536854</v>
+        <v>14.5149296121117</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
@@ -4418,28 +4392,28 @@
         <v>24</v>
       </c>
       <c r="B25">
-        <v>2.0319E-2</v>
+        <v>0</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>1.36283347597763E-2</v>
+        <v>2.92209159481092E-4</v>
       </c>
       <c r="E25">
-        <v>6.4276456827220899E-2</v>
+        <v>2.93651791905402E-3</v>
       </c>
       <c r="F25">
-        <v>7.7579808235168501</v>
+        <v>0</v>
       </c>
       <c r="G25">
         <v>0</v>
       </c>
       <c r="H25">
-        <v>5.2000386928772997</v>
+        <v>0.10742366010604699</v>
       </c>
       <c r="I25">
-        <v>23.5923497014136</v>
+        <v>1.1567882328129699</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
@@ -4447,28 +4421,28 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>1.7330000000000002E-2</v>
+        <v>0</v>
       </c>
       <c r="C26">
-        <v>7.49532040452982E-3</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>1.1794350521588301E-2</v>
+        <v>0</v>
       </c>
       <c r="E26">
-        <v>2.41924867131709E-2</v>
+        <v>6.32838562994192E-4</v>
       </c>
       <c r="F26">
-        <v>83.645599365234403</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>57.366487667290102</v>
+        <v>0</v>
       </c>
       <c r="H26">
-        <v>73.175308044668796</v>
+        <v>0</v>
       </c>
       <c r="I26">
-        <v>89.754487135175495</v>
+        <v>4.8654239616742103</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
@@ -4482,101 +4456,22 @@
         <v>0</v>
       </c>
       <c r="D27">
-        <v>0</v>
+        <v>4.7809732811758001E-4</v>
       </c>
       <c r="E27">
-        <v>1.6210979352312201E-2</v>
+        <v>4.4067916057889097E-3</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>9.9772647023201003E-2</v>
       </c>
       <c r="G27">
         <v>0</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>0.39614942847127899</v>
       </c>
       <c r="I27">
-        <v>12.3726032489385</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7719C31F-8C86-2A48-A332-856CE760E1A9}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="3" max="3" width="21.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="C2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="C3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1">
-        <v>0.39</v>
-      </c>
-      <c r="C4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1">
-        <v>0.27</v>
-      </c>
-      <c r="C5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="C6" t="s">
-        <v>42</v>
+        <v>3.4195987140228898</v>
       </c>
     </row>
   </sheetData>

</xml_diff>